<commit_message>
Lot « Chicoutimi / Jonquière » : 10 personnages (183 → 193), 6 rues nouvelles, garde-fou géographique
- data/personnages.csv : 6 personnages à Chicoutimi (rues Bossé,
  Jacques-Cartier Ouest, Sainte-Anne, du Havre) et 4 à Jonquière (rue Davis
  à Arvida, Saint-Hubert, rue du Vieux-Pont), rues réelles OSM (Nominatim).
  Répartition : La Baie 143 / Chicoutimi 34 / Jonquière 16.
- portraits/ : 10 portraits IA 3:2, gabarits -web et -vignette (184-193).
- Livrables régénérés ; construction idempotente.
- tests : N = 193, test_les_deux_autres_arrondissements_restent_peuples
  (planchers d'effectif et de rues) → 40 garde-fous ; README, CHANGELOG.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/base_personnages_fictifs.xlsx
+++ b/base_personnages_fictifs.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Lisez-moi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Personnages'!$A$1:$P$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Personnages'!$A$1:$P$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P184"/>
+  <dimension ref="A1:P194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -11467,12 +11467,12 @@
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>Gilles Dufour</t>
+          <t>Gaétan Bossé</t>
         </is>
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>Monsieur le Maire</t>
+          <t>Le Bouquiniste</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
@@ -11481,11 +11481,11 @@
         </is>
       </c>
       <c r="D153" s="6" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>Maire de Saguenay</t>
+          <t>Bouquiniste — livres usagés</t>
         </is>
       </c>
       <c r="F153" s="5" t="inlineStr">
@@ -11495,69 +11495,69 @@
       </c>
       <c r="G153" s="5" t="inlineStr">
         <is>
-          <t>201, Rue Racine Est</t>
+          <t>312, Rue Bossé</t>
         </is>
       </c>
       <c r="H153" s="7" t="n">
-        <v>48.4282</v>
+        <v>48.42445</v>
       </c>
       <c r="I153" s="7" t="n">
-        <v>-71.0534</v>
+        <v>-71.07605</v>
       </c>
       <c r="J153" s="5" t="inlineStr">
         <is>
-          <t>Cheveux gris, veston marine</t>
+          <t>Barbe grise, lunettes sur le front</t>
         </is>
       </c>
       <c r="K153" s="5" t="inlineStr">
         <is>
-          <t>Complet, épinglette de ville</t>
+          <t>Veste de laine sur chemise à carreaux</t>
         </is>
       </c>
       <c r="L153" s="5" t="inlineStr">
         <is>
-          <t>Poignée de main</t>
+          <t>Livre relié sous le bras</t>
         </is>
       </c>
       <c r="M153" s="5" t="inlineStr">
         <is>
-          <t>portraits/121-gilles-dufour-web.webp</t>
+          <t>portraits/184-gaetan-bosse-web.webp</t>
         </is>
       </c>
       <c r="N153" s="5" t="inlineStr">
         <is>
-          <t>Dufour</t>
-        </is>
-      </c>
-      <c r="O153" s="5" t="inlineStr">
-        <is>
-          <t>hôtel de ville</t>
-        </is>
-      </c>
+          <t>Bossé</t>
+        </is>
+      </c>
+      <c r="O153" s="5" t="n"/>
       <c r="P153" s="5" t="inlineStr">
         <is>
-          <t>Fils d’Albert Dufour — maire de Saguenay</t>
+          <t>Frère de Stéphane Bossé</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Hélène Samson</t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="n"/>
+          <t>Gilles Dufour</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Monsieur le Maire</t>
+        </is>
+      </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D154" s="3" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Retraitée — ex-secrétaire de palais</t>
+          <t>Maire de Saguenay</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -11567,51 +11567,55 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>149, Rue Bégin</t>
+          <t>201, Rue Racine Est</t>
         </is>
       </c>
       <c r="H154" s="4" t="n">
-        <v>48.4213</v>
+        <v>48.4282</v>
       </c>
       <c r="I154" s="4" t="n">
-        <v>-71.0574</v>
+        <v>-71.0534</v>
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>Cheveux soignés, manteau beige</t>
+          <t>Cheveux gris, veston marine</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
-          <t>Manteau beige</t>
+          <t>Complet, épinglette de ville</t>
         </is>
       </c>
       <c r="L154" s="2" t="inlineStr">
         <is>
-          <t>Sac à main</t>
+          <t>Poignée de main</t>
         </is>
       </c>
       <c r="M154" s="2" t="inlineStr">
         <is>
-          <t>portraits/168-helene-samson-web.webp</t>
+          <t>portraits/121-gilles-dufour-web.webp</t>
         </is>
       </c>
       <c r="N154" s="2" t="inlineStr">
         <is>
-          <t>Samson</t>
-        </is>
-      </c>
-      <c r="O154" s="2" t="n"/>
+          <t>Dufour</t>
+        </is>
+      </c>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>hôtel de ville</t>
+        </is>
+      </c>
       <c r="P154" s="2" t="inlineStr">
         <is>
-          <t>Mère de Pierre Samson</t>
+          <t>Fils d’Albert Dufour — maire de Saguenay</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>Isabelle Gagné</t>
+          <t>Hélène Samson</t>
         </is>
       </c>
       <c r="B155" s="5" t="n"/>
@@ -11621,11 +11625,11 @@
         </is>
       </c>
       <c r="D155" s="6" t="n">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>Députée — Assemblée nationale</t>
+          <t>Retraitée — ex-secrétaire de palais</t>
         </is>
       </c>
       <c r="F155" s="5" t="inlineStr">
@@ -11635,73 +11639,65 @@
       </c>
       <c r="G155" s="5" t="inlineStr">
         <is>
-          <t>145, Rue Racine Est</t>
+          <t>149, Rue Bégin</t>
         </is>
       </c>
       <c r="H155" s="7" t="n">
-        <v>48.4279</v>
+        <v>48.4213</v>
       </c>
       <c r="I155" s="7" t="n">
-        <v>-71.0531</v>
+        <v>-71.0574</v>
       </c>
       <c r="J155" s="5" t="inlineStr">
         <is>
-          <t>Carré blond, blazer rouge</t>
+          <t>Cheveux soignés, manteau beige</t>
         </is>
       </c>
       <c r="K155" s="5" t="inlineStr">
         <is>
-          <t>Blazer rouge</t>
+          <t>Manteau beige</t>
         </is>
       </c>
       <c r="L155" s="5" t="inlineStr">
         <is>
-          <t>Épinglette fleurdelisé</t>
+          <t>Sac à main</t>
         </is>
       </c>
       <c r="M155" s="5" t="inlineStr">
         <is>
-          <t>portraits/122-isabelle-gagne-web.webp</t>
+          <t>portraits/168-helene-samson-web.webp</t>
         </is>
       </c>
       <c r="N155" s="5" t="inlineStr">
         <is>
-          <t>Gagné</t>
-        </is>
-      </c>
-      <c r="O155" s="5" t="inlineStr">
-        <is>
-          <t>politique</t>
-        </is>
-      </c>
+          <t>Samson</t>
+        </is>
+      </c>
+      <c r="O155" s="5" t="n"/>
       <c r="P155" s="5" t="inlineStr">
         <is>
-          <t>Célibataire</t>
+          <t>Mère de Pierre Samson</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Roy</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>Johnny Fake</t>
-        </is>
-      </c>
+          <t>Isabelle Gagné</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="n"/>
       <c r="C156" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D156" s="3" t="n">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>Arnaqueur — fausses identités</t>
+          <t>Députée — Assemblée nationale</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
@@ -11711,60 +11707,60 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>1186, Boulevard Talbot</t>
+          <t>145, Rue Racine Est</t>
         </is>
       </c>
       <c r="H156" s="4" t="n">
-        <v>48.3986</v>
+        <v>48.4279</v>
       </c>
       <c r="I156" s="4" t="n">
-        <v>-71.0675</v>
+        <v>-71.0531</v>
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>Cheveux gominés, sourire</t>
+          <t>Carré blond, blazer rouge</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>Complet cheap</t>
+          <t>Blazer rouge</t>
         </is>
       </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>Trois cellulaires</t>
+          <t>Épinglette fleurdelisé</t>
         </is>
       </c>
       <c r="M156" s="2" t="inlineStr">
         <is>
-          <t>portraits/119-jonathan-roy-web.webp</t>
+          <t>portraits/122-isabelle-gagne-web.webp</t>
         </is>
       </c>
       <c r="N156" s="2" t="inlineStr">
         <is>
-          <t>Roy</t>
+          <t>Gagné</t>
         </is>
       </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
-          <t>arnaque</t>
+          <t>politique</t>
         </is>
       </c>
       <c r="P156" s="2" t="inlineStr">
         <is>
-          <t>Célibataire — croise Alex Tremblay</t>
+          <t>Célibataire</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>Julien Gagné</t>
+          <t>Jonathan Roy</t>
         </is>
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>Le Volant</t>
+          <t>Johnny Fake</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
@@ -11773,11 +11769,11 @@
         </is>
       </c>
       <c r="D157" s="6" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>Chauffeur de voiture de ville</t>
+          <t>Arnaqueur — fausses identités</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
@@ -11787,56 +11783,60 @@
       </c>
       <c r="G157" s="5" t="inlineStr">
         <is>
-          <t>1188, Boulevard Talbot</t>
+          <t>1186, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H157" s="7" t="n">
-        <v>48.3983</v>
+        <v>48.3986</v>
       </c>
       <c r="I157" s="7" t="n">
-        <v>-71.06780000000001</v>
+        <v>-71.0675</v>
       </c>
       <c r="J157" s="5" t="inlineStr">
         <is>
-          <t>Complet noir, oreillette</t>
+          <t>Cheveux gominés, sourire</t>
         </is>
       </c>
       <c r="K157" s="5" t="inlineStr">
         <is>
-          <t>Complet noir</t>
+          <t>Complet cheap</t>
         </is>
       </c>
       <c r="L157" s="5" t="inlineStr">
         <is>
-          <t>VUS noir</t>
+          <t>Trois cellulaires</t>
         </is>
       </c>
       <c r="M157" s="5" t="inlineStr">
         <is>
-          <t>portraits/157-julien-gagne-web.webp</t>
+          <t>portraits/119-jonathan-roy-web.webp</t>
         </is>
       </c>
       <c r="N157" s="5" t="inlineStr">
         <is>
-          <t>Santini</t>
-        </is>
-      </c>
-      <c r="O157" s="5" t="n"/>
+          <t>Roy</t>
+        </is>
+      </c>
+      <c r="O157" s="5" t="inlineStr">
+        <is>
+          <t>arnaque</t>
+        </is>
+      </c>
       <c r="P157" s="5" t="inlineStr">
         <is>
-          <t>Chauffeur de Vittorio</t>
+          <t>Célibataire — croise Alex Tremblay</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Justin Chen</t>
+          <t>Julien Gagné</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Junior Talbot</t>
+          <t>Le Volant</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
@@ -11845,11 +11845,11 @@
         </is>
       </c>
       <c r="D158" s="3" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Étudiant en administration (Cégep de Chicoutimi)</t>
+          <t>Chauffeur de voiture de ville</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -11859,65 +11859,69 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>1180, Boulevard Talbot</t>
+          <t>1188, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H158" s="4" t="n">
-        <v>48.398223</v>
+        <v>48.3983</v>
       </c>
       <c r="I158" s="4" t="n">
-        <v>-71.06763599999999</v>
+        <v>-71.06780000000001</v>
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>Métis, Moncler propre</t>
+          <t>Complet noir, oreillette</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
-          <t>Moncler noir</t>
+          <t>Complet noir</t>
         </is>
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>Paye trop cher</t>
+          <t>VUS noir</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>portraits/26-justin-chen-web.webp</t>
+          <t>portraits/157-julien-gagne-web.webp</t>
         </is>
       </c>
       <c r="N158" s="2" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Santini</t>
         </is>
       </c>
       <c r="O158" s="2" t="n"/>
       <c r="P158" s="2" t="inlineStr">
         <is>
-          <t>Fils de Mei</t>
+          <t>Chauffeur de Vittorio</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>Laurie Lavoie</t>
-        </is>
-      </c>
-      <c r="B159" s="5" t="n"/>
+          <t>Justin Chen</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Junior Talbot</t>
+        </is>
+      </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D159" s="6" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>Étudiante en psychologie (UQAC)</t>
+          <t>Étudiant en administration (Cégep de Chicoutimi)</t>
         </is>
       </c>
       <c r="F159" s="5" t="inlineStr">
@@ -11927,69 +11931,69 @@
       </c>
       <c r="G159" s="5" t="inlineStr">
         <is>
-          <t>555, Boulevard de l'Université</t>
+          <t>1180, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H159" s="7" t="n">
-        <v>48.421623</v>
+        <v>48.398223</v>
       </c>
       <c r="I159" s="7" t="n">
-        <v>-71.07566199999999</v>
+        <v>-71.06763599999999</v>
       </c>
       <c r="J159" s="5" t="inlineStr">
         <is>
-          <t>Cheveux longs châtains, hoodie UQAC</t>
+          <t>Métis, Moncler propre</t>
         </is>
       </c>
       <c r="K159" s="5" t="inlineStr">
         <is>
-          <t>Hoodie UQAC</t>
+          <t>Moncler noir</t>
         </is>
       </c>
       <c r="L159" s="5" t="inlineStr">
         <is>
-          <t>Livre psycho</t>
+          <t>Paye trop cher</t>
         </is>
       </c>
       <c r="M159" s="5" t="inlineStr">
         <is>
-          <t>portraits/36-laurie-lavoie-web.webp</t>
+          <t>portraits/26-justin-chen-web.webp</t>
         </is>
       </c>
       <c r="N159" s="5" t="inlineStr">
         <is>
-          <t>Lavoie</t>
-        </is>
-      </c>
-      <c r="O159" s="5" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="O159" s="5" t="n"/>
       <c r="P159" s="5" t="inlineStr">
         <is>
-          <t>Sœur de JP</t>
+          <t>Fils de Mei</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Louise Villeneuve</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="n"/>
+          <t>Jérémie Côté</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Ti-Poste</t>
+        </is>
+      </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D160" s="3" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Juge — Cour du Québec</t>
+          <t>Facteur — Postes Canada</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
@@ -11999,73 +12003,69 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>227, Rue Racine Est</t>
+          <t>145, Rue Sainte-Anne</t>
         </is>
       </c>
       <c r="H160" s="4" t="n">
-        <v>48.4275</v>
+        <v>48.42915</v>
       </c>
       <c r="I160" s="4" t="n">
-        <v>-71.05419999999999</v>
+        <v>-71.06835</v>
       </c>
       <c r="J160" s="2" t="inlineStr">
         <is>
-          <t>Regard sévère, toge</t>
+          <t>Barbe taillée, joues rouges</t>
         </is>
       </c>
       <c r="K160" s="2" t="inlineStr">
         <is>
-          <t>Toge</t>
+          <t>Parka de facteur à bandes</t>
         </is>
       </c>
       <c r="L160" s="2" t="inlineStr">
         <is>
-          <t>Marteau de bois</t>
+          <t>Sacoche de courrier</t>
         </is>
       </c>
       <c r="M160" s="2" t="inlineStr">
         <is>
-          <t>portraits/127-louise-villeneuve-web.webp</t>
+          <t>portraits/187-jeremie-cote-web.webp</t>
         </is>
       </c>
       <c r="N160" s="2" t="inlineStr">
         <is>
-          <t>Villeneuve</t>
+          <t>Côté</t>
         </is>
       </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
-          <t>palais</t>
+          <t>poste</t>
         </is>
       </c>
       <c r="P160" s="2" t="inlineStr">
         <is>
-          <t>Collègue de Catherine Samson</t>
+          <t>Neveu d’Alain Côté</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>Maria Santini</t>
-        </is>
-      </c>
-      <c r="B161" s="5" t="inlineStr">
-        <is>
-          <t>Donna Maria</t>
-        </is>
-      </c>
+          <t>Laurie Lavoie</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="n"/>
       <c r="C161" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D161" s="6" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>Matriarche — restaurant familial</t>
+          <t>Étudiante en psychologie (UQAC)</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
@@ -12075,51 +12075,55 @@
       </c>
       <c r="G161" s="5" t="inlineStr">
         <is>
-          <t>200, Rue Racine Est</t>
+          <t>555, Boulevard de l'Université</t>
         </is>
       </c>
       <c r="H161" s="7" t="n">
-        <v>48.42815</v>
+        <v>48.421623</v>
       </c>
       <c r="I161" s="7" t="n">
-        <v>-71.0543</v>
+        <v>-71.07566199999999</v>
       </c>
       <c r="J161" s="5" t="inlineStr">
         <is>
-          <t>Cheveux sombres, perles</t>
+          <t>Cheveux longs châtains, hoodie UQAC</t>
         </is>
       </c>
       <c r="K161" s="5" t="inlineStr">
         <is>
-          <t>Robe noire</t>
+          <t>Hoodie UQAC</t>
         </is>
       </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
-          <t>Rosaire au poignet</t>
+          <t>Livre psycho</t>
         </is>
       </c>
       <c r="M161" s="5" t="inlineStr">
         <is>
-          <t>portraits/152-maria-santini-web.webp</t>
+          <t>portraits/36-laurie-lavoie-web.webp</t>
         </is>
       </c>
       <c r="N161" s="5" t="inlineStr">
         <is>
-          <t>Santini</t>
-        </is>
-      </c>
-      <c r="O161" s="5" t="n"/>
+          <t>Lavoie</t>
+        </is>
+      </c>
+      <c r="O161" s="5" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
       <c r="P161" s="5" t="inlineStr">
         <is>
-          <t>Épouse de Vittorio</t>
+          <t>Sœur de JP</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Mei Chen</t>
+          <t>Lise Gauthier</t>
         </is>
       </c>
       <c r="B162" s="2" t="n"/>
@@ -12129,11 +12133,11 @@
         </is>
       </c>
       <c r="D162" s="3" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Préposée d’hôtel</t>
+          <t>Infirmière clinicienne — CLSC</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
@@ -12143,69 +12147,65 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>1182, Boulevard Talbot</t>
+          <t>222, Rue du Havre</t>
         </is>
       </c>
       <c r="H162" s="4" t="n">
-        <v>48.39835</v>
+        <v>48.4293</v>
       </c>
       <c r="I162" s="4" t="n">
-        <v>-71.06775</v>
+        <v>-71.05445</v>
       </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
-          <t>Chinoise, chignon, calme</t>
+          <t>Cheveux blancs courts, lunettes à chaînette</t>
         </is>
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>Uniforme hôtel</t>
+          <t>Cardigan bourgogne sur uniforme</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>Badges de chambre</t>
+          <t>Tensiomètre</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr">
         <is>
-          <t>portraits/63-mei-chen-web.webp</t>
+          <t>portraits/188-lise-gauthier-web.webp</t>
         </is>
       </c>
       <c r="N162" s="2" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Gauthier</t>
         </is>
       </c>
       <c r="O162" s="2" t="n"/>
       <c r="P162" s="2" t="inlineStr">
         <is>
-          <t>Mère de Justin Chen</t>
+          <t>Tante de Steve et Chantal Gauthier</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>Mgr Paul Tremblay</t>
-        </is>
-      </c>
-      <c r="B163" s="5" t="inlineStr">
-        <is>
-          <t>Monseigneur</t>
-        </is>
-      </c>
+          <t>Louise Villeneuve</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="n"/>
       <c r="C163" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D163" s="6" t="n">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>Évêque — diocèse de Chicoutimi</t>
+          <t>Juge — Cour du Québec</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
@@ -12215,60 +12215,60 @@
       </c>
       <c r="G163" s="5" t="inlineStr">
         <is>
-          <t>602, Rue Racine Est</t>
+          <t>227, Rue Racine Est</t>
         </is>
       </c>
       <c r="H163" s="7" t="n">
-        <v>48.4268</v>
+        <v>48.4275</v>
       </c>
       <c r="I163" s="7" t="n">
-        <v>-71.0538</v>
+        <v>-71.05419999999999</v>
       </c>
       <c r="J163" s="5" t="inlineStr">
         <is>
-          <t>Cheveux blancs, col romain</t>
+          <t>Regard sévère, toge</t>
         </is>
       </c>
       <c r="K163" s="5" t="inlineStr">
         <is>
-          <t>Soutane, rabat violet</t>
+          <t>Toge</t>
         </is>
       </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
-          <t>Anneau pastoral</t>
+          <t>Marteau de bois</t>
         </is>
       </c>
       <c r="M163" s="5" t="inlineStr">
         <is>
-          <t>portraits/126-mgr-paul-tremblay-web.webp</t>
+          <t>portraits/127-louise-villeneuve-web.webp</t>
         </is>
       </c>
       <c r="N163" s="5" t="inlineStr">
         <is>
-          <t>Tremblay</t>
+          <t>Villeneuve</t>
         </is>
       </c>
       <c r="O163" s="5" t="inlineStr">
         <is>
-          <t>Église</t>
+          <t>palais</t>
         </is>
       </c>
       <c r="P163" s="5" t="inlineStr">
         <is>
-          <t>Supérieur de Lucien Lacroix</t>
+          <t>Collègue de Catherine Samson</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Nico Santini</t>
+          <t>Maria Santini</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Nico</t>
+          <t>Donna Maria</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -12277,11 +12277,11 @@
         </is>
       </c>
       <c r="D164" s="3" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Préposé à la sécurité — restaurant</t>
+          <t>Matriarche — restaurant familial</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -12291,33 +12291,33 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>202, Rue Racine Est</t>
+          <t>200, Rue Racine Est</t>
         </is>
       </c>
       <c r="H164" s="4" t="n">
-        <v>48.4282</v>
+        <v>48.42815</v>
       </c>
       <c r="I164" s="4" t="n">
-        <v>-71.05459999999999</v>
+        <v>-71.0543</v>
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
-          <t>Cheveux gominés, veste cuir</t>
+          <t>Cheveux sombres, perles</t>
         </is>
       </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
-          <t>Veste de cuir</t>
+          <t>Robe noire</t>
         </is>
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>Sourire de défi</t>
+          <t>Rosaire au poignet</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>portraits/160-nico-santini-web.webp</t>
+          <t>portraits/152-maria-santini-web.webp</t>
         </is>
       </c>
       <c r="N164" s="2" t="inlineStr">
@@ -12328,17 +12328,21 @@
       <c r="O164" s="2" t="n"/>
       <c r="P164" s="2" t="inlineStr">
         <is>
-          <t>Fils de Vittorio et Maria</t>
+          <t>Épouse de Vittorio</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>Olivier Savard</t>
-        </is>
-      </c>
-      <c r="B165" s="5" t="n"/>
+          <t>Marie-Ève Boucher</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>La Plume</t>
+        </is>
+      </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
@@ -12349,7 +12353,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>Journaliste — Le Quotidien</t>
+          <t>Journaliste — quotidien régional</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
@@ -12359,69 +12363,65 @@
       </c>
       <c r="G165" s="5" t="inlineStr">
         <is>
-          <t>100, Rue Racine Est</t>
+          <t>412, Rue Jacques-Cartier Ouest</t>
         </is>
       </c>
       <c r="H165" s="7" t="n">
-        <v>48.4278</v>
+        <v>48.4268</v>
       </c>
       <c r="I165" s="7" t="n">
-        <v>-71.05289999999999</v>
+        <v>-71.0699</v>
       </c>
       <c r="J165" s="5" t="inlineStr">
         <is>
-          <t>Barbe, sacoche</t>
+          <t>Cheveux courts noirs, regard vif</t>
         </is>
       </c>
       <c r="K165" s="5" t="inlineStr">
         <is>
-          <t>Manteau de ville</t>
+          <t>Trench, cordon de presse</t>
         </is>
       </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
-          <t>Carnet spiralé</t>
+          <t>Calepin et téléphone</t>
         </is>
       </c>
       <c r="M165" s="5" t="inlineStr">
         <is>
-          <t>portraits/78-olivier-savard-web.webp</t>
+          <t>portraits/185-marie-eve-boucher-web.webp</t>
         </is>
       </c>
       <c r="N165" s="5" t="inlineStr">
         <is>
-          <t>Savard</t>
+          <t>Bossé</t>
         </is>
       </c>
       <c r="O165" s="5" t="n"/>
       <c r="P165" s="5" t="inlineStr">
         <is>
-          <t>Célibataire — ex-collègue de JP</t>
+          <t>Conjointe de Stéphane Bossé — cousine de Normand Boucher</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Patrick Lapointe</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>Pat</t>
-        </is>
-      </c>
+          <t>Mei Chen</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="n"/>
       <c r="C166" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D166" s="3" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneur en construction</t>
+          <t>Préposée d’hôtel</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -12431,60 +12431,56 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>1250, Boulevard Talbot</t>
+          <t>1182, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H166" s="4" t="n">
-        <v>48.3985</v>
+        <v>48.39835</v>
       </c>
       <c r="I166" s="4" t="n">
-        <v>-71.06276</v>
+        <v>-71.06775</v>
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
-          <t>Polo construction</t>
+          <t>Chinoise, chignon, calme</t>
         </is>
       </c>
       <c r="K166" s="2" t="inlineStr">
         <is>
-          <t>Polo construction</t>
+          <t>Uniforme hôtel</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>Devis 400k</t>
+          <t>Badges de chambre</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr">
         <is>
-          <t>portraits/39-patrick-lapointe-web.webp</t>
+          <t>portraits/63-mei-chen-web.webp</t>
         </is>
       </c>
       <c r="N166" s="2" t="inlineStr">
         <is>
-          <t>Lapointe</t>
-        </is>
-      </c>
-      <c r="O166" s="2" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="O166" s="2" t="n"/>
       <c r="P166" s="2" t="inlineStr">
         <is>
-          <t>Frère de Marco</t>
+          <t>Mère de Justin Chen</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>Paul-André Côté</t>
+          <t>Mgr Paul Tremblay</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
         <is>
-          <t>Le Chiffre</t>
+          <t>Monseigneur</t>
         </is>
       </c>
       <c r="C167" s="6" t="inlineStr">
@@ -12493,11 +12489,11 @@
         </is>
       </c>
       <c r="D167" s="6" t="n">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>Comptable — sociétés-écrans</t>
+          <t>Évêque — diocèse de Chicoutimi</t>
         </is>
       </c>
       <c r="F167" s="5" t="inlineStr">
@@ -12507,56 +12503,60 @@
       </c>
       <c r="G167" s="5" t="inlineStr">
         <is>
-          <t>1252, Boulevard Talbot</t>
+          <t>602, Rue Racine Est</t>
         </is>
       </c>
       <c r="H167" s="7" t="n">
-        <v>48.39855</v>
+        <v>48.4268</v>
       </c>
       <c r="I167" s="7" t="n">
-        <v>-71.0629</v>
+        <v>-71.0538</v>
       </c>
       <c r="J167" s="5" t="inlineStr">
         <is>
-          <t>Maigre, lunettes cheap</t>
+          <t>Cheveux blancs, col romain</t>
         </is>
       </c>
       <c r="K167" s="5" t="inlineStr">
         <is>
-          <t>Chemise et classeur</t>
+          <t>Soutane, rabat violet</t>
         </is>
       </c>
       <c r="L167" s="5" t="inlineStr">
         <is>
-          <t>Tableurs</t>
+          <t>Anneau pastoral</t>
         </is>
       </c>
       <c r="M167" s="5" t="inlineStr">
         <is>
-          <t>portraits/156-paul-andre-cote-web.webp</t>
+          <t>portraits/126-mgr-paul-tremblay-web.webp</t>
         </is>
       </c>
       <c r="N167" s="5" t="inlineStr">
         <is>
-          <t>Santini</t>
-        </is>
-      </c>
-      <c r="O167" s="5" t="n"/>
+          <t>Tremblay</t>
+        </is>
+      </c>
+      <c r="O167" s="5" t="inlineStr">
+        <is>
+          <t>Église</t>
+        </is>
+      </c>
       <c r="P167" s="5" t="inlineStr">
         <is>
-          <t>Comptable du clan — croise Bertrand Gagnon</t>
+          <t>Supérieur de Lucien Lacroix</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Pierre Samson</t>
+          <t>Nico Santini</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>L'Enquêteur</t>
+          <t>Nico</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -12565,11 +12565,11 @@
         </is>
       </c>
       <c r="D168" s="3" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Policier — Service de police de Saguenay, stupéfiants</t>
+          <t>Préposé à la sécurité — restaurant</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -12579,69 +12579,65 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>145, Rue Bégin</t>
+          <t>202, Rue Racine Est</t>
         </is>
       </c>
       <c r="H168" s="4" t="n">
-        <v>48.421205</v>
+        <v>48.4282</v>
       </c>
       <c r="I168" s="4" t="n">
-        <v>-71.057355</v>
+        <v>-71.05459999999999</v>
       </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
-          <t>Cernes violacés</t>
+          <t>Cheveux gominés, veste cuir</t>
         </is>
       </c>
       <c r="K168" s="2" t="inlineStr">
         <is>
-          <t>Pardessus brun-beige</t>
+          <t>Veste de cuir</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>Clique Bic bleu</t>
+          <t>Sourire de défi</t>
         </is>
       </c>
       <c r="M168" s="2" t="inlineStr">
         <is>
-          <t>portraits/07-pierre-samson-web.webp</t>
+          <t>portraits/160-nico-santini-web.webp</t>
         </is>
       </c>
       <c r="N168" s="2" t="inlineStr">
         <is>
-          <t>Samson</t>
+          <t>Santini</t>
         </is>
       </c>
       <c r="O168" s="2" t="n"/>
       <c r="P168" s="2" t="inlineStr">
         <is>
-          <t>Fils d’Hélène Samson — époux de Catherine</t>
+          <t>Fils de Vittorio et Maria</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>Sofia Santini</t>
-        </is>
-      </c>
-      <c r="B169" s="5" t="inlineStr">
-        <is>
-          <t>Sofi</t>
-        </is>
-      </c>
+          <t>Olivier Savard</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="n"/>
       <c r="C169" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D169" s="6" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>Élève du secondaire — aide au restaurant familial</t>
+          <t>Journaliste — Le Quotidien</t>
         </is>
       </c>
       <c r="F169" s="5" t="inlineStr">
@@ -12651,65 +12647,69 @@
       </c>
       <c r="G169" s="5" t="inlineStr">
         <is>
-          <t>204, Rue Racine Est</t>
+          <t>100, Rue Racine Est</t>
         </is>
       </c>
       <c r="H169" s="7" t="n">
-        <v>48.42825</v>
+        <v>48.4278</v>
       </c>
       <c r="I169" s="7" t="n">
-        <v>-71.05475</v>
+        <v>-71.05289999999999</v>
       </c>
       <c r="J169" s="5" t="inlineStr">
         <is>
-          <t>Cheveux noirs ondulés, sourire en coin</t>
+          <t>Barbe, sacoche</t>
         </is>
       </c>
       <c r="K169" s="5" t="inlineStr">
         <is>
-          <t>Tablier noir de service</t>
+          <t>Manteau de ville</t>
         </is>
       </c>
       <c r="L169" s="5" t="inlineStr">
         <is>
-          <t>Cabaret à deux mains</t>
+          <t>Carnet spiralé</t>
         </is>
       </c>
       <c r="M169" s="5" t="inlineStr">
         <is>
-          <t>portraits/177-sofia-santini-web.webp</t>
+          <t>portraits/78-olivier-savard-web.webp</t>
         </is>
       </c>
       <c r="N169" s="5" t="inlineStr">
         <is>
-          <t>Santini</t>
+          <t>Savard</t>
         </is>
       </c>
       <c r="O169" s="5" t="n"/>
       <c r="P169" s="5" t="inlineStr">
         <is>
-          <t>Fille de Nico Santini — petite-fille de Vittorio et Maria</t>
+          <t>Célibataire — ex-collègue de JP</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Sophie Labbé</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="n"/>
+          <t>Patrick Lapointe</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Pat</t>
+        </is>
+      </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D170" s="3" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>Psychologue — clinique UQAC</t>
+          <t>Entrepreneur en construction</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -12719,56 +12719,60 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>555, Boulevard de l'Université</t>
+          <t>1250, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H170" s="4" t="n">
-        <v>48.4215</v>
+        <v>48.3985</v>
       </c>
       <c r="I170" s="4" t="n">
-        <v>-71.07550000000001</v>
+        <v>-71.06276</v>
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>Chignon, lunettes</t>
+          <t>Polo construction</t>
         </is>
       </c>
       <c r="K170" s="2" t="inlineStr">
         <is>
-          <t>Cardigan</t>
+          <t>Polo construction</t>
         </is>
       </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
-          <t>Carnet de notes</t>
+          <t>Devis 400k</t>
         </is>
       </c>
       <c r="M170" s="2" t="inlineStr">
         <is>
-          <t>portraits/104-sophie-labbe-web.webp</t>
+          <t>portraits/39-patrick-lapointe-web.webp</t>
         </is>
       </c>
       <c r="N170" s="2" t="inlineStr">
         <is>
-          <t>Labbé</t>
-        </is>
-      </c>
-      <c r="O170" s="2" t="n"/>
+          <t>Lapointe</t>
+        </is>
+      </c>
+      <c r="O170" s="2" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
       <c r="P170" s="2" t="inlineStr">
         <is>
-          <t>Célibataire — collègue de Laurie Lavoie</t>
+          <t>Frère de Marco</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="inlineStr">
         <is>
-          <t>Vittorio Santini</t>
+          <t>Paul-André Côté</t>
         </is>
       </c>
       <c r="B171" s="5" t="inlineStr">
         <is>
-          <t>Don Vittorio</t>
+          <t>Le Chiffre</t>
         </is>
       </c>
       <c r="C171" s="6" t="inlineStr">
@@ -12777,11 +12781,11 @@
         </is>
       </c>
       <c r="D171" s="6" t="n">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>Homme d’affaires — restauration et bars</t>
+          <t>Comptable — sociétés-écrans</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
@@ -12791,33 +12795,33 @@
       </c>
       <c r="G171" s="5" t="inlineStr">
         <is>
-          <t>200, Rue Racine Est</t>
+          <t>1252, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H171" s="7" t="n">
-        <v>48.4281</v>
+        <v>48.39855</v>
       </c>
       <c r="I171" s="7" t="n">
-        <v>-71.0545</v>
+        <v>-71.0629</v>
       </c>
       <c r="J171" s="5" t="inlineStr">
         <is>
-          <t>Cheveux argentés gominés, chevalière</t>
+          <t>Maigre, lunettes cheap</t>
         </is>
       </c>
       <c r="K171" s="5" t="inlineStr">
         <is>
-          <t>Manteau noir</t>
+          <t>Chemise et classeur</t>
         </is>
       </c>
       <c r="L171" s="5" t="inlineStr">
         <is>
-          <t>Chevalière en or</t>
+          <t>Tableurs</t>
         </is>
       </c>
       <c r="M171" s="5" t="inlineStr">
         <is>
-          <t>portraits/151-vittorio-santini-web.webp</t>
+          <t>portraits/156-paul-andre-cote-web.webp</t>
         </is>
       </c>
       <c r="N171" s="5" t="inlineStr">
@@ -12828,19 +12832,19 @@
       <c r="O171" s="5" t="n"/>
       <c r="P171" s="5" t="inlineStr">
         <is>
-          <t>Époux de Maria — tient Dévon à distance</t>
+          <t>Comptable du clan — croise Bertrand Gagnon</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Éric Simard</t>
+          <t>Pierre Samson</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Ti-Eric</t>
+          <t>L'Enquêteur</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -12849,11 +12853,11 @@
         </is>
       </c>
       <c r="D172" s="3" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>Étudiant — Cégep de Chicoutimi</t>
+          <t>Policier — Service de police de Saguenay, stupéfiants</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
@@ -12863,56 +12867,56 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>1184, Boulevard Talbot</t>
+          <t>145, Rue Bégin</t>
         </is>
       </c>
       <c r="H172" s="4" t="n">
-        <v>48.3984</v>
+        <v>48.421205</v>
       </c>
       <c r="I172" s="4" t="n">
-        <v>-71.06740000000001</v>
+        <v>-71.057355</v>
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>Casquette, jeans</t>
+          <t>Cernes violacés</t>
         </is>
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>Hoodie cégep</t>
+          <t>Pardessus brun-beige</t>
         </is>
       </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
-          <t>Skateboard</t>
+          <t>Clique Bic bleu</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr">
         <is>
-          <t>portraits/100-eric-simard-web.webp</t>
+          <t>portraits/07-pierre-samson-web.webp</t>
         </is>
       </c>
       <c r="N172" s="2" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Samson</t>
         </is>
       </c>
       <c r="O172" s="2" t="n"/>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>Colocataire de Justin Chen</t>
+          <t>Fils d’Hélène Samson — époux de Catherine</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>Antoine Lefèvre</t>
+          <t>Sofia Santini</t>
         </is>
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Le Français</t>
+          <t>Sofi</t>
         </is>
       </c>
       <c r="C173" s="6" t="inlineStr">
@@ -12921,65 +12925,65 @@
         </is>
       </c>
       <c r="D173" s="6" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+          <t>Élève du secondaire — aide au restaurant familial</t>
         </is>
       </c>
       <c r="F173" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>1125, Rue Saint-Dominique</t>
+          <t>204, Rue Racine Est</t>
         </is>
       </c>
       <c r="H173" s="7" t="n">
-        <v>48.421279</v>
+        <v>48.42825</v>
       </c>
       <c r="I173" s="7" t="n">
-        <v>-71.244586</v>
+        <v>-71.05475</v>
       </c>
       <c r="J173" s="5" t="inlineStr">
         <is>
-          <t>Barbe hipster</t>
+          <t>Cheveux noirs ondulés, sourire en coin</t>
         </is>
       </c>
       <c r="K173" s="5" t="inlineStr">
         <is>
-          <t>Friperie, caméra Sony</t>
+          <t>Tablier noir de service</t>
         </is>
       </c>
       <c r="L173" s="5" t="inlineStr">
         <is>
-          <t>Veut docu raw</t>
+          <t>Cabaret à deux mains</t>
         </is>
       </c>
       <c r="M173" s="5" t="inlineStr">
         <is>
-          <t>portraits/20-antoine-lefevre-web.webp</t>
+          <t>portraits/177-sofia-santini-web.webp</t>
         </is>
       </c>
       <c r="N173" s="5" t="inlineStr">
         <is>
-          <t>Lefèvre</t>
+          <t>Santini</t>
         </is>
       </c>
       <c r="O173" s="5" t="n"/>
       <c r="P173" s="5" t="inlineStr">
         <is>
-          <t>Frère de Camille</t>
+          <t>Fille de Nico Santini — petite-fille de Vittorio et Maria</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Benoit Larouche</t>
+          <t>Sophie Labbé</t>
         </is>
       </c>
       <c r="B174" s="2" t="n"/>
@@ -12989,133 +12993,137 @@
         </is>
       </c>
       <c r="D174" s="3" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>Enseignant — Cégep de Jonquière (ATM)</t>
+          <t>Psychologue — clinique UQAC</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>2505, Rue Saint-Hubert</t>
+          <t>555, Boulevard de l'Université</t>
         </is>
       </c>
       <c r="H174" s="4" t="n">
-        <v>48.416</v>
+        <v>48.4215</v>
       </c>
       <c r="I174" s="4" t="n">
-        <v>-71.253</v>
+        <v>-71.07550000000001</v>
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>Lunettes, barbe grise</t>
+          <t>Chignon, lunettes</t>
         </is>
       </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
-          <t>Chemise et cardigan</t>
+          <t>Cardigan</t>
         </is>
       </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
-          <t>Clap de cinéma</t>
+          <t>Carnet de notes</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr">
         <is>
-          <t>portraits/86-benoit-larouche-web.webp</t>
+          <t>portraits/104-sophie-labbe-web.webp</t>
         </is>
       </c>
       <c r="N174" s="2" t="inlineStr">
         <is>
-          <t>Larouche</t>
+          <t>Labbé</t>
         </is>
       </c>
       <c r="O174" s="2" t="n"/>
       <c r="P174" s="2" t="inlineStr">
         <is>
-          <t>Prof d’Antoine Lefèvre</t>
+          <t>Célibataire — collègue de Laurie Lavoie</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>Camille Lefèvre</t>
-        </is>
-      </c>
-      <c r="B175" s="5" t="n"/>
+          <t>Stéphane Bossé</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Steph Patate</t>
+        </is>
+      </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D175" s="6" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>Étudiante en communications (UQAC)</t>
+          <t>Cuisinier — casse-croûte</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>1127, Rue Saint-Dominique</t>
+          <t>410, Rue Jacques-Cartier Ouest</t>
         </is>
       </c>
       <c r="H175" s="7" t="n">
-        <v>48.4214</v>
+        <v>48.42675</v>
       </c>
       <c r="I175" s="7" t="n">
-        <v>-71.24469999999999</v>
+        <v>-71.07004999999999</v>
       </c>
       <c r="J175" s="5" t="inlineStr">
         <is>
-          <t>Carré brun, appareil photo</t>
+          <t>Cheveux ras, avant-bras tatoués</t>
         </is>
       </c>
       <c r="K175" s="5" t="inlineStr">
         <is>
-          <t>Manteau friperie</t>
+          <t>Tablier blanc taché</t>
         </is>
       </c>
       <c r="L175" s="5" t="inlineStr">
         <is>
-          <t>Pentax vintage</t>
+          <t>Spatule à la main</t>
         </is>
       </c>
       <c r="M175" s="5" t="inlineStr">
         <is>
-          <t>portraits/65-camille-lefevre-web.webp</t>
+          <t>portraits/186-stephane-bosse-web.webp</t>
         </is>
       </c>
       <c r="N175" s="5" t="inlineStr">
         <is>
-          <t>Lefèvre</t>
+          <t>Bossé</t>
         </is>
       </c>
       <c r="O175" s="5" t="n"/>
       <c r="P175" s="5" t="inlineStr">
         <is>
-          <t>Sœur d’Antoine Lefèvre</t>
+          <t>Frère de Gaétan Bossé — conjoint de Marie-Ève Boucher</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Dany Aubin</t>
+          <t>Valentina Rojas</t>
         </is>
       </c>
       <c r="B176" s="2" t="n"/>
@@ -13125,70 +13133,70 @@
         </is>
       </c>
       <c r="D176" s="3" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>Soudeur</t>
+          <t>Épicière — produits latino-américains</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>2147, Boulevard Harvey</t>
+          <t>318, Rue Bossé</t>
         </is>
       </c>
       <c r="H176" s="4" t="n">
-        <v>48.41282</v>
+        <v>48.4245</v>
       </c>
       <c r="I176" s="4" t="n">
-        <v>-71.24145</v>
+        <v>-71.07585</v>
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>Brûlé de soudeur, casque relevé</t>
+          <t>Longs cheveux noirs, anneaux dorés</t>
         </is>
       </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
-          <t>Manteau de soudeur</t>
+          <t>Tablier vert sur chandail</t>
         </is>
       </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
-          <t>Masque de soudure</t>
+          <t>Caisse de plantains</t>
         </is>
       </c>
       <c r="M176" s="2" t="inlineStr">
         <is>
-          <t>portraits/66-dany-aubin-web.webp</t>
+          <t>portraits/189-valentina-rojas-web.webp</t>
         </is>
       </c>
       <c r="N176" s="2" t="inlineStr">
         <is>
-          <t>Aubin</t>
+          <t>Rojas</t>
         </is>
       </c>
       <c r="O176" s="2" t="n"/>
       <c r="P176" s="2" t="inlineStr">
         <is>
-          <t>Frère de Sam Aubin</t>
+          <t>Célibataire</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>Gérald Tremblay</t>
+          <t>Vittorio Santini</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
         <is>
-          <t>Le Syndic</t>
+          <t>Don Vittorio</t>
         </is>
       </c>
       <c r="C177" s="6" t="inlineStr">
@@ -13197,151 +13205,155 @@
         </is>
       </c>
       <c r="D177" s="6" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="E177" s="5" t="inlineStr">
         <is>
-          <t>Délégué syndical — aluminerie</t>
+          <t>Homme d’affaires — restauration et bars</t>
         </is>
       </c>
       <c r="F177" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G177" s="5" t="inlineStr">
         <is>
-          <t>3324, Rue Price</t>
+          <t>200, Rue Racine Est</t>
         </is>
       </c>
       <c r="H177" s="7" t="n">
-        <v>48.4258</v>
+        <v>48.4281</v>
       </c>
       <c r="I177" s="7" t="n">
-        <v>-71.24039999999999</v>
+        <v>-71.0545</v>
       </c>
       <c r="J177" s="5" t="inlineStr">
         <is>
-          <t>Manteau de travail, épinglette</t>
+          <t>Cheveux argentés gominés, chevalière</t>
         </is>
       </c>
       <c r="K177" s="5" t="inlineStr">
         <is>
-          <t>Manteau d’usine</t>
+          <t>Manteau noir</t>
         </is>
       </c>
       <c r="L177" s="5" t="inlineStr">
         <is>
-          <t>Cartable de griefs</t>
+          <t>Chevalière en or</t>
         </is>
       </c>
       <c r="M177" s="5" t="inlineStr">
         <is>
-          <t>portraits/137-gerald-tremblay-web.webp</t>
+          <t>portraits/151-vittorio-santini-web.webp</t>
         </is>
       </c>
       <c r="N177" s="5" t="inlineStr">
         <is>
-          <t>Tremblay</t>
-        </is>
-      </c>
-      <c r="O177" s="5" t="inlineStr">
-        <is>
-          <t>syndicat</t>
-        </is>
-      </c>
+          <t>Santini</t>
+        </is>
+      </c>
+      <c r="O177" s="5" t="n"/>
       <c r="P177" s="5" t="inlineStr">
         <is>
-          <t>Collègue de Mathieu Lavoie</t>
+          <t>Époux de Maria — tient Dévon à distance</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Jade Boivin</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="n"/>
+          <t>Éric Simard</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Ti-Eric</t>
+        </is>
+      </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D178" s="3" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>Élève du primaire — patineuse artistique</t>
+          <t>Étudiant — Cégep de Chicoutimi</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>2350, Rue Sainte-Famille</t>
+          <t>1184, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H178" s="4" t="n">
-        <v>48.4293</v>
+        <v>48.3984</v>
       </c>
       <c r="I178" s="4" t="n">
-        <v>-71.23480000000001</v>
+        <v>-71.06740000000001</v>
       </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>Chignon serré, sourire édenté</t>
+          <t>Casquette, jeans</t>
         </is>
       </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
-          <t>Veston d’entraînement mauve</t>
+          <t>Hoodie cégep</t>
         </is>
       </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
-          <t>Protège-lames</t>
+          <t>Skateboard</t>
         </is>
       </c>
       <c r="M178" s="2" t="inlineStr">
         <is>
-          <t>portraits/183-jade-boivin-web.webp</t>
+          <t>portraits/100-eric-simard-web.webp</t>
         </is>
       </c>
       <c r="N178" s="2" t="inlineStr">
         <is>
-          <t>Boivin</t>
+          <t>Chen</t>
         </is>
       </c>
       <c r="O178" s="2" t="n"/>
       <c r="P178" s="2" t="inlineStr">
         <is>
-          <t>Nièce de France et Maxime Boivin</t>
+          <t>Colocataire de Justin Chen</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
         <is>
-          <t>Jean-Marc Fortin</t>
-        </is>
-      </c>
-      <c r="B179" s="5" t="n"/>
+          <t>Antoine Lefèvre</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Le Français</t>
+        </is>
+      </c>
       <c r="C179" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D179" s="6" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>Directeur d’usine — Rio Tinto Arvida</t>
+          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
@@ -13351,73 +13363,65 @@
       </c>
       <c r="G179" s="5" t="inlineStr">
         <is>
-          <t>1, Rue des Alumineries</t>
+          <t>1125, Rue Saint-Dominique</t>
         </is>
       </c>
       <c r="H179" s="7" t="n">
-        <v>48.4265</v>
+        <v>48.421279</v>
       </c>
       <c r="I179" s="7" t="n">
-        <v>-71.182</v>
+        <v>-71.244586</v>
       </c>
       <c r="J179" s="5" t="inlineStr">
         <is>
-          <t>Cheveux argentés, manteau</t>
+          <t>Barbe hipster</t>
         </is>
       </c>
       <c r="K179" s="5" t="inlineStr">
         <is>
-          <t>Manteau et casque blanc</t>
+          <t>Friperie, caméra Sony</t>
         </is>
       </c>
       <c r="L179" s="5" t="inlineStr">
         <is>
-          <t>Casque sous le bras</t>
+          <t>Veut docu raw</t>
         </is>
       </c>
       <c r="M179" s="5" t="inlineStr">
         <is>
-          <t>portraits/125-jean-marc-fortin-web.webp</t>
+          <t>portraits/20-antoine-lefevre-web.webp</t>
         </is>
       </c>
       <c r="N179" s="5" t="inlineStr">
         <is>
-          <t>Fortin</t>
-        </is>
-      </c>
-      <c r="O179" s="5" t="inlineStr">
-        <is>
-          <t>industrie</t>
-        </is>
-      </c>
+          <t>Lefèvre</t>
+        </is>
+      </c>
+      <c r="O179" s="5" t="n"/>
       <c r="P179" s="5" t="inlineStr">
         <is>
-          <t>Patron de Mathieu Lavoie et Nicolas Gagné</t>
+          <t>Frère de Camille</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Ludovic Larouche</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>Ludo</t>
-        </is>
-      </c>
+          <t>Audrey Lavoie</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="n"/>
       <c r="C180" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D180" s="3" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+          <t>Apprentie électricienne — aluminerie Rio Tinto Arvida</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -13427,69 +13431,69 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>2507, Rue Saint-Hubert</t>
+          <t>2135, Rue Davis</t>
         </is>
       </c>
       <c r="H180" s="4" t="n">
-        <v>48.41615</v>
+        <v>48.42455</v>
       </c>
       <c r="I180" s="4" t="n">
-        <v>-71.25285</v>
+        <v>-71.18219999999999</v>
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>Boucles, lunettes rondes</t>
+          <t>Tresse blonde, lunettes de sécurité</t>
         </is>
       </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
-          <t>Veste en velours côtelé</t>
+          <t>Manteau orange haute visibilité</t>
         </is>
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>Caméscope à l’épaule</t>
+          <t>Glacière à lunch</t>
         </is>
       </c>
       <c r="M180" s="2" t="inlineStr">
         <is>
-          <t>portraits/182-ludovic-larouche-web.webp</t>
+          <t>portraits/191-audrey-lavoie-web.webp</t>
         </is>
       </c>
       <c r="N180" s="2" t="inlineStr">
         <is>
-          <t>Larouche</t>
-        </is>
-      </c>
-      <c r="O180" s="2" t="n"/>
+          <t>Lavoie</t>
+        </is>
+      </c>
+      <c r="O180" s="2" t="inlineStr">
+        <is>
+          <t>Arvida</t>
+        </is>
+      </c>
       <c r="P180" s="2" t="inlineStr">
         <is>
-          <t>Fils de Benoit Larouche</t>
+          <t>Fille de Fernand Lavoie — collègue de Nicolas Gagné</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="inlineStr">
         <is>
-          <t>Mathieu Lavoie</t>
-        </is>
-      </c>
-      <c r="B181" s="5" t="inlineStr">
-        <is>
-          <t>Mat</t>
-        </is>
-      </c>
+          <t>Benoit Larouche</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="n"/>
       <c r="C181" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D181" s="6" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>Technicien à l'aluminerie Rio Tinto — Arvida</t>
+          <t>Enseignant — Cégep de Jonquière (ATM)</t>
         </is>
       </c>
       <c r="F181" s="5" t="inlineStr">
@@ -13499,55 +13503,51 @@
       </c>
       <c r="G181" s="5" t="inlineStr">
         <is>
-          <t>3320, Rue Price</t>
+          <t>2505, Rue Saint-Hubert</t>
         </is>
       </c>
       <c r="H181" s="7" t="n">
-        <v>48.425907</v>
+        <v>48.416</v>
       </c>
       <c r="I181" s="7" t="n">
-        <v>-71.240752</v>
+        <v>-71.253</v>
       </c>
       <c r="J181" s="5" t="inlineStr">
         <is>
-          <t>Propre, polo Rio Tinto</t>
+          <t>Lunettes, barbe grise</t>
         </is>
       </c>
       <c r="K181" s="5" t="inlineStr">
         <is>
-          <t>Polo Rio Tinto</t>
+          <t>Chemise et cardigan</t>
         </is>
       </c>
       <c r="L181" s="5" t="inlineStr">
         <is>
-          <t>Boîte à lunch</t>
+          <t>Clap de cinéma</t>
         </is>
       </c>
       <c r="M181" s="5" t="inlineStr">
         <is>
-          <t>portraits/35-mathieu-lavoie-web.webp</t>
+          <t>portraits/86-benoit-larouche-web.webp</t>
         </is>
       </c>
       <c r="N181" s="5" t="inlineStr">
         <is>
-          <t>Lavoie</t>
-        </is>
-      </c>
-      <c r="O181" s="5" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
+          <t>Larouche</t>
+        </is>
+      </c>
+      <c r="O181" s="5" t="n"/>
       <c r="P181" s="5" t="inlineStr">
         <is>
-          <t>Frère aîné de JP</t>
+          <t>Prof d’Antoine Lefèvre</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Mélissa Harvey</t>
+          <t>Camille Lefèvre</t>
         </is>
       </c>
       <c r="B182" s="2" t="n"/>
@@ -13561,7 +13561,7 @@
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>Étudiante en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+          <t>Étudiante en communications (UQAC)</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -13571,18 +13571,18 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>1129, Rue Saint-Dominique</t>
+          <t>1127, Rue Saint-Dominique</t>
         </is>
       </c>
       <c r="H182" s="4" t="n">
-        <v>48.42135</v>
+        <v>48.4214</v>
       </c>
       <c r="I182" s="4" t="n">
-        <v>-71.24464999999999</v>
+        <v>-71.24469999999999</v>
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>Chignon brouillon, manteau friperie</t>
+          <t>Carré brun, appareil photo</t>
         </is>
       </c>
       <c r="K182" s="2" t="inlineStr">
@@ -13592,30 +13592,30 @@
       </c>
       <c r="L182" s="2" t="inlineStr">
         <is>
-          <t>Perche micro</t>
+          <t>Pentax vintage</t>
         </is>
       </c>
       <c r="M182" s="2" t="inlineStr">
         <is>
-          <t>portraits/110-melissa-harvey-web.webp</t>
+          <t>portraits/65-camille-lefevre-web.webp</t>
         </is>
       </c>
       <c r="N182" s="2" t="inlineStr">
         <is>
-          <t>Harvey</t>
+          <t>Lefèvre</t>
         </is>
       </c>
       <c r="O182" s="2" t="n"/>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>Nièce de François Harvey</t>
+          <t>Sœur d’Antoine Lefèvre</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="inlineStr">
         <is>
-          <t>Nicolas Gagné</t>
+          <t>Dany Aubin</t>
         </is>
       </c>
       <c r="B183" s="5" t="n"/>
@@ -13625,11 +13625,11 @@
         </is>
       </c>
       <c r="D183" s="6" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>Technicien — aluminerie Rio Tinto Arvida</t>
+          <t>Soudeur</t>
         </is>
       </c>
       <c r="F183" s="5" t="inlineStr">
@@ -13639,125 +13639,849 @@
       </c>
       <c r="G183" s="5" t="inlineStr">
         <is>
-          <t>3322, Rue Price</t>
+          <t>2147, Boulevard Harvey</t>
         </is>
       </c>
       <c r="H183" s="7" t="n">
-        <v>48.426</v>
+        <v>48.41282</v>
       </c>
       <c r="I183" s="7" t="n">
-        <v>-71.2405</v>
+        <v>-71.24145</v>
       </c>
       <c r="J183" s="5" t="inlineStr">
         <is>
-          <t>Propre, lunettes de sécurité</t>
+          <t>Brûlé de soudeur, casque relevé</t>
         </is>
       </c>
       <c r="K183" s="5" t="inlineStr">
         <is>
-          <t>Polo Rio Tinto</t>
+          <t>Manteau de soudeur</t>
         </is>
       </c>
       <c r="L183" s="5" t="inlineStr">
         <is>
-          <t>Casque blanc</t>
+          <t>Masque de soudure</t>
         </is>
       </c>
       <c r="M183" s="5" t="inlineStr">
         <is>
-          <t>portraits/94-nicolas-gagne-web.webp</t>
+          <t>portraits/66-dany-aubin-web.webp</t>
         </is>
       </c>
       <c r="N183" s="5" t="inlineStr">
         <is>
-          <t>Gagné</t>
-        </is>
-      </c>
-      <c r="O183" s="5" t="inlineStr">
-        <is>
-          <t>Arvida</t>
-        </is>
-      </c>
+          <t>Aubin</t>
+        </is>
+      </c>
+      <c r="O183" s="5" t="n"/>
       <c r="P183" s="5" t="inlineStr">
         <is>
-          <t>Collègue de Mathieu Lavoie</t>
+          <t>Frère de Sam Aubin</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
+          <t>Fernand Lavoie</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Ti-Fer</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>Retraité — ex-opérateur de cuves à l’aluminerie</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>2131, Rue Davis</t>
+        </is>
+      </c>
+      <c r="H184" s="4" t="n">
+        <v>48.4244</v>
+      </c>
+      <c r="I184" s="4" t="n">
+        <v>-71.18225</v>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>Casquette plate, mains larges</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Veste de laine à carreaux</t>
+        </is>
+      </c>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>Pipe éteinte</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>portraits/190-fernand-lavoie-web.webp</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="inlineStr">
+        <is>
+          <t>Lavoie</t>
+        </is>
+      </c>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>Arvida</t>
+        </is>
+      </c>
+      <c r="P184" s="2" t="inlineStr">
+        <is>
+          <t>Père d’Audrey Lavoie — cousin éloigné de Mathieu Lavoie</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>Gérald Tremblay</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Le Syndic</t>
+        </is>
+      </c>
+      <c r="C185" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D185" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>Délégué syndical — aluminerie</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>3324, Rue Price</t>
+        </is>
+      </c>
+      <c r="H185" s="7" t="n">
+        <v>48.4258</v>
+      </c>
+      <c r="I185" s="7" t="n">
+        <v>-71.24039999999999</v>
+      </c>
+      <c r="J185" s="5" t="inlineStr">
+        <is>
+          <t>Manteau de travail, épinglette</t>
+        </is>
+      </c>
+      <c r="K185" s="5" t="inlineStr">
+        <is>
+          <t>Manteau d’usine</t>
+        </is>
+      </c>
+      <c r="L185" s="5" t="inlineStr">
+        <is>
+          <t>Cartable de griefs</t>
+        </is>
+      </c>
+      <c r="M185" s="5" t="inlineStr">
+        <is>
+          <t>portraits/137-gerald-tremblay-web.webp</t>
+        </is>
+      </c>
+      <c r="N185" s="5" t="inlineStr">
+        <is>
+          <t>Tremblay</t>
+        </is>
+      </c>
+      <c r="O185" s="5" t="inlineStr">
+        <is>
+          <t>syndicat</t>
+        </is>
+      </c>
+      <c r="P185" s="5" t="inlineStr">
+        <is>
+          <t>Collègue de Mathieu Lavoie</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Jade Boivin</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="n"/>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>Élève du primaire — patineuse artistique</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>2350, Rue Sainte-Famille</t>
+        </is>
+      </c>
+      <c r="H186" s="4" t="n">
+        <v>48.4293</v>
+      </c>
+      <c r="I186" s="4" t="n">
+        <v>-71.23480000000001</v>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>Chignon serré, sourire édenté</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>Veston d’entraînement mauve</t>
+        </is>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>Protège-lames</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>portraits/183-jade-boivin-web.webp</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="inlineStr">
+        <is>
+          <t>Boivin</t>
+        </is>
+      </c>
+      <c r="O186" s="2" t="n"/>
+      <c r="P186" s="2" t="inlineStr">
+        <is>
+          <t>Nièce de France et Maxime Boivin</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>Jean-Marc Fortin</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="n"/>
+      <c r="C187" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D187" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>Directeur d’usine — Rio Tinto Arvida</t>
+        </is>
+      </c>
+      <c r="F187" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>1, Rue des Alumineries</t>
+        </is>
+      </c>
+      <c r="H187" s="7" t="n">
+        <v>48.4265</v>
+      </c>
+      <c r="I187" s="7" t="n">
+        <v>-71.182</v>
+      </c>
+      <c r="J187" s="5" t="inlineStr">
+        <is>
+          <t>Cheveux argentés, manteau</t>
+        </is>
+      </c>
+      <c r="K187" s="5" t="inlineStr">
+        <is>
+          <t>Manteau et casque blanc</t>
+        </is>
+      </c>
+      <c r="L187" s="5" t="inlineStr">
+        <is>
+          <t>Casque sous le bras</t>
+        </is>
+      </c>
+      <c r="M187" s="5" t="inlineStr">
+        <is>
+          <t>portraits/125-jean-marc-fortin-web.webp</t>
+        </is>
+      </c>
+      <c r="N187" s="5" t="inlineStr">
+        <is>
+          <t>Fortin</t>
+        </is>
+      </c>
+      <c r="O187" s="5" t="inlineStr">
+        <is>
+          <t>industrie</t>
+        </is>
+      </c>
+      <c r="P187" s="5" t="inlineStr">
+        <is>
+          <t>Patron de Mathieu Lavoie et Nicolas Gagné</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Ludovic Larouche</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Ludo</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>2507, Rue Saint-Hubert</t>
+        </is>
+      </c>
+      <c r="H188" s="4" t="n">
+        <v>48.41615</v>
+      </c>
+      <c r="I188" s="4" t="n">
+        <v>-71.25285</v>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>Boucles, lunettes rondes</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>Veste en velours côtelé</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>Caméscope à l’épaule</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>portraits/182-ludovic-larouche-web.webp</t>
+        </is>
+      </c>
+      <c r="N188" s="2" t="inlineStr">
+        <is>
+          <t>Larouche</t>
+        </is>
+      </c>
+      <c r="O188" s="2" t="n"/>
+      <c r="P188" s="2" t="inlineStr">
+        <is>
+          <t>Fils de Benoit Larouche</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>Marc Picard</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>L’Arpenteur</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D189" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>Arpenteur-géomètre</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>1220, Rue du Vieux-Pont</t>
+        </is>
+      </c>
+      <c r="H189" s="7" t="n">
+        <v>48.4113</v>
+      </c>
+      <c r="I189" s="7" t="n">
+        <v>-71.2679</v>
+      </c>
+      <c r="J189" s="5" t="inlineStr">
+        <is>
+          <t>Innu de Mashteuiatsh, cheveux longs attachés</t>
+        </is>
+      </c>
+      <c r="K189" s="5" t="inlineStr">
+        <is>
+          <t>Dossard orange sur polar</t>
+        </is>
+      </c>
+      <c r="L189" s="5" t="inlineStr">
+        <is>
+          <t>Station totale sur trépied</t>
+        </is>
+      </c>
+      <c r="M189" s="5" t="inlineStr">
+        <is>
+          <t>portraits/193-marc-picard-web.webp</t>
+        </is>
+      </c>
+      <c r="N189" s="5" t="inlineStr">
+        <is>
+          <t>Picard</t>
+        </is>
+      </c>
+      <c r="O189" s="5" t="n"/>
+      <c r="P189" s="5" t="inlineStr">
+        <is>
+          <t>Célibataire — croise William McKenzie</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Mathieu Lavoie</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>Technicien à l'aluminerie Rio Tinto — Arvida</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>3320, Rue Price</t>
+        </is>
+      </c>
+      <c r="H190" s="4" t="n">
+        <v>48.425907</v>
+      </c>
+      <c r="I190" s="4" t="n">
+        <v>-71.240752</v>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>Propre, polo Rio Tinto</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>Polo Rio Tinto</t>
+        </is>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>Boîte à lunch</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>portraits/35-mathieu-lavoie-web.webp</t>
+        </is>
+      </c>
+      <c r="N190" s="2" t="inlineStr">
+        <is>
+          <t>Lavoie</t>
+        </is>
+      </c>
+      <c r="O190" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="P190" s="2" t="inlineStr">
+        <is>
+          <t>Frère aîné de JP</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>Mélissa Harvey</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="n"/>
+      <c r="C191" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D191" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>Étudiante en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>1129, Rue Saint-Dominique</t>
+        </is>
+      </c>
+      <c r="H191" s="7" t="n">
+        <v>48.42135</v>
+      </c>
+      <c r="I191" s="7" t="n">
+        <v>-71.24464999999999</v>
+      </c>
+      <c r="J191" s="5" t="inlineStr">
+        <is>
+          <t>Chignon brouillon, manteau friperie</t>
+        </is>
+      </c>
+      <c r="K191" s="5" t="inlineStr">
+        <is>
+          <t>Manteau friperie</t>
+        </is>
+      </c>
+      <c r="L191" s="5" t="inlineStr">
+        <is>
+          <t>Perche micro</t>
+        </is>
+      </c>
+      <c r="M191" s="5" t="inlineStr">
+        <is>
+          <t>portraits/110-melissa-harvey-web.webp</t>
+        </is>
+      </c>
+      <c r="N191" s="5" t="inlineStr">
+        <is>
+          <t>Harvey</t>
+        </is>
+      </c>
+      <c r="O191" s="5" t="n"/>
+      <c r="P191" s="5" t="inlineStr">
+        <is>
+          <t>Nièce de François Harvey</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Nancy Simard</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Nancy Ciseaux</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>Coiffeuse — propriétaire de salon</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>3812, Rue Saint-Hubert</t>
+        </is>
+      </c>
+      <c r="H192" s="4" t="n">
+        <v>48.41605</v>
+      </c>
+      <c r="I192" s="4" t="n">
+        <v>-71.2453</v>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>Blond platine, grosses boucles d’oreilles</t>
+        </is>
+      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>Sarrau noir de coiffeuse</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>Ciseaux et peigne</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>portraits/192-nancy-simard-web.webp</t>
+        </is>
+      </c>
+      <c r="N192" s="2" t="inlineStr">
+        <is>
+          <t>Simard</t>
+        </is>
+      </c>
+      <c r="O192" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="P192" s="2" t="inlineStr">
+        <is>
+          <t>Célibataire — voisine de Benoit Larouche</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>Nicolas Gagné</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="n"/>
+      <c r="C193" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D193" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>Technicien — aluminerie Rio Tinto Arvida</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>3322, Rue Price</t>
+        </is>
+      </c>
+      <c r="H193" s="7" t="n">
+        <v>48.426</v>
+      </c>
+      <c r="I193" s="7" t="n">
+        <v>-71.2405</v>
+      </c>
+      <c r="J193" s="5" t="inlineStr">
+        <is>
+          <t>Propre, lunettes de sécurité</t>
+        </is>
+      </c>
+      <c r="K193" s="5" t="inlineStr">
+        <is>
+          <t>Polo Rio Tinto</t>
+        </is>
+      </c>
+      <c r="L193" s="5" t="inlineStr">
+        <is>
+          <t>Casque blanc</t>
+        </is>
+      </c>
+      <c r="M193" s="5" t="inlineStr">
+        <is>
+          <t>portraits/94-nicolas-gagne-web.webp</t>
+        </is>
+      </c>
+      <c r="N193" s="5" t="inlineStr">
+        <is>
+          <t>Gagné</t>
+        </is>
+      </c>
+      <c r="O193" s="5" t="inlineStr">
+        <is>
+          <t>Arvida</t>
+        </is>
+      </c>
+      <c r="P193" s="5" t="inlineStr">
+        <is>
+          <t>Collègue de Mathieu Lavoie</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
           <t>Sam Aubin</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
+      <c r="B194" s="2" t="inlineStr">
         <is>
           <t>Ink</t>
         </is>
       </c>
-      <c r="C184" s="3" t="inlineStr">
-        <is>
-          <t>Humain</t>
-        </is>
-      </c>
-      <c r="D184" s="3" t="n">
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="E184" s="2" t="inlineStr">
+      <c r="E194" s="2" t="inlineStr">
         <is>
           <t>Tatoueur</t>
         </is>
       </c>
-      <c r="F184" s="2" t="inlineStr">
+      <c r="F194" s="2" t="inlineStr">
         <is>
           <t>Jonquière</t>
         </is>
       </c>
-      <c r="G184" s="2" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
         <is>
           <t>2145, Boulevard Harvey</t>
         </is>
       </c>
-      <c r="H184" s="4" t="n">
+      <c r="H194" s="4" t="n">
         <v>48.412694</v>
       </c>
-      <c r="I184" s="4" t="n">
+      <c r="I194" s="4" t="n">
         <v>-71.241325</v>
       </c>
-      <c r="J184" s="2" t="inlineStr">
+      <c r="J194" s="2" t="inlineStr">
         <is>
           <t>Cheveux bleus, full tattoos</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr">
+      <c r="K194" s="2" t="inlineStr">
         <is>
           <t>Tablier noir</t>
         </is>
       </c>
-      <c r="L184" s="2" t="inlineStr">
+      <c r="L194" s="2" t="inlineStr">
         <is>
           <t>Efface tattoos gang</t>
         </is>
       </c>
-      <c r="M184" s="2" t="inlineStr">
+      <c r="M194" s="2" t="inlineStr">
         <is>
           <t>portraits/24-sam-aubin-web.webp</t>
         </is>
       </c>
-      <c r="N184" s="2" t="inlineStr">
+      <c r="N194" s="2" t="inlineStr">
         <is>
           <t>Aubin</t>
         </is>
       </c>
-      <c r="O184" s="2" t="n"/>
-      <c r="P184" s="2" t="inlineStr">
+      <c r="O194" s="2" t="n"/>
+      <c r="P194" s="2" t="inlineStr">
         <is>
           <t>Frère de Dany</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P184"/>
+  <autoFilter ref="A1:P194"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13793,7 +14517,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>183 entrées · 16 colonnes · région du Saguenay (Québec)</t>
+          <t>193 entrées · 16 colonnes · région du Saguenay (Québec)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lot « Cégep / UQAC et Kénogami » : 10 personnages (203 → 213), lot mixte jeunes/encadrants
- data/personnages.csv : colocation étudiante du 318 Saint-Vallier
  (Chicoutimi) + propriétaire, jeunes autour du cégep (LaFontaine, Dréan),
  foyer Simard/Kénogami (rue Saint-Joseph, Jonquière) — rues réelles OSM.
  Moins de 25 ans : 10,4 % → 13,2 % ; La Baie 153 / Chicoutimi 41 / Jonquière 19.
- portraits 204-213 (IA, 3:2), livrables régénérés, construction idempotente.
- tests : N = 213, MINEURS + Léa Simard ; README, CHANGELOG.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/base_personnages_fictifs.xlsx
+++ b/base_personnages_fictifs.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Lisez-moi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Personnages'!$A$1:$P$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Personnages'!$A$1:$P$214</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P204"/>
+  <dimension ref="A1:P214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -12055,12 +12055,12 @@
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>Enzo Bianchi</t>
+          <t>Diane Perron</t>
         </is>
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Le Conseiller</t>
+          <t>La Prof</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
@@ -12069,11 +12069,11 @@
         </is>
       </c>
       <c r="D161" s="6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>Conseiller en gestion d’entreprise</t>
+          <t>Professeure de sociologie (UQAC)</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
@@ -12083,65 +12083,69 @@
       </c>
       <c r="G161" s="5" t="inlineStr">
         <is>
-          <t>198, Rue Racine Est</t>
+          <t>126, Rue Dréan</t>
         </is>
       </c>
       <c r="H161" s="7" t="n">
-        <v>48.428</v>
+        <v>48.42605</v>
       </c>
       <c r="I161" s="7" t="n">
-        <v>-71.05419999999999</v>
+        <v>-71.0804</v>
       </c>
       <c r="J161" s="5" t="inlineStr">
         <is>
-          <t>Lunettes, complet gris</t>
+          <t>Longs cheveux gris, boucles d’oreilles en argent</t>
         </is>
       </c>
       <c r="K161" s="5" t="inlineStr">
         <is>
-          <t>Complet gris</t>
+          <t>Blazer de lin sur col roulé</t>
         </is>
       </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
-          <t>Carnet de cuir</t>
+          <t>Pile de copies</t>
         </is>
       </c>
       <c r="M161" s="5" t="inlineStr">
         <is>
-          <t>portraits/153-enzo-bianchi-web.webp</t>
+          <t>portraits/209-diane-perron-web.webp</t>
         </is>
       </c>
       <c r="N161" s="5" t="inlineStr">
         <is>
-          <t>Santini</t>
+          <t>Perron</t>
         </is>
       </c>
       <c r="O161" s="5" t="n"/>
       <c r="P161" s="5" t="inlineStr">
         <is>
-          <t>Conseiller de Vittorio</t>
+          <t>Célibataire — directrice de recherche de Laurie Lavoie</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>François Côté</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="n"/>
+          <t>Emma Boucher</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Em</t>
+        </is>
+      </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D162" s="3" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Rédacteur en chef — Le Quotidien</t>
+          <t>Étudiante en sciences humaines (Cégep de Chicoutimi)</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
@@ -12151,60 +12155,60 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>100, Rue Racine Est</t>
+          <t>318, Rue Saint-Vallier</t>
         </is>
       </c>
       <c r="H162" s="4" t="n">
-        <v>48.4277</v>
+        <v>48.42635</v>
       </c>
       <c r="I162" s="4" t="n">
-        <v>-71.053</v>
+        <v>-71.05029999999999</v>
       </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
-          <t>Manches relevées, stylo rouge</t>
+          <t>Cheveux mauves, lunettes</t>
         </is>
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>Chemise de rédaction</t>
+          <t>Gros tricot</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>Stylo rouge</t>
+          <t>Portable couvert d’autocollants</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr">
         <is>
-          <t>portraits/134-francois-cote-web.webp</t>
+          <t>portraits/204-emma-boucher-web.webp</t>
         </is>
       </c>
       <c r="N162" s="2" t="inlineStr">
         <is>
-          <t>Côté</t>
+          <t>Boucher</t>
         </is>
       </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
-          <t>presse</t>
+          <t>coloc</t>
         </is>
       </c>
       <c r="P162" s="2" t="inlineStr">
         <is>
-          <t>Patron d’Olivier Savard — ex-patron de JP</t>
+          <t>Nièce de Fernande Boucher — cousine de Dévon — colocataire de Moussa et William</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
         <is>
-          <t>Gaétan Bossé</t>
+          <t>Enzo Bianchi</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Le Bouquiniste</t>
+          <t>Le Conseiller</t>
         </is>
       </c>
       <c r="C163" s="6" t="inlineStr">
@@ -12213,11 +12217,11 @@
         </is>
       </c>
       <c r="D163" s="6" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>Bouquiniste — livres usagés</t>
+          <t>Conseiller en gestion d’entreprise</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
@@ -12227,69 +12231,65 @@
       </c>
       <c r="G163" s="5" t="inlineStr">
         <is>
-          <t>312, Rue Bossé</t>
+          <t>198, Rue Racine Est</t>
         </is>
       </c>
       <c r="H163" s="7" t="n">
-        <v>48.42445</v>
+        <v>48.428</v>
       </c>
       <c r="I163" s="7" t="n">
-        <v>-71.07605</v>
+        <v>-71.05419999999999</v>
       </c>
       <c r="J163" s="5" t="inlineStr">
         <is>
-          <t>Barbe grise, lunettes sur le front</t>
+          <t>Lunettes, complet gris</t>
         </is>
       </c>
       <c r="K163" s="5" t="inlineStr">
         <is>
-          <t>Veste de laine sur chemise à carreaux</t>
+          <t>Complet gris</t>
         </is>
       </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
-          <t>Livre relié sous le bras</t>
+          <t>Carnet de cuir</t>
         </is>
       </c>
       <c r="M163" s="5" t="inlineStr">
         <is>
-          <t>portraits/184-gaetan-bosse-web.webp</t>
+          <t>portraits/153-enzo-bianchi-web.webp</t>
         </is>
       </c>
       <c r="N163" s="5" t="inlineStr">
         <is>
-          <t>Bossé</t>
+          <t>Santini</t>
         </is>
       </c>
       <c r="O163" s="5" t="n"/>
       <c r="P163" s="5" t="inlineStr">
         <is>
-          <t>Frère de Stéphane Bossé</t>
+          <t>Conseiller de Vittorio</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Gilles Dufour</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>Monsieur le Maire</t>
-        </is>
-      </c>
+          <t>François Côté</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="n"/>
       <c r="C164" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D164" s="3" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Maire de Saguenay</t>
+          <t>Rédacteur en chef — Le Quotidien</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -12299,69 +12299,73 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>201, Rue Racine Est</t>
+          <t>100, Rue Racine Est</t>
         </is>
       </c>
       <c r="H164" s="4" t="n">
-        <v>48.4282</v>
+        <v>48.4277</v>
       </c>
       <c r="I164" s="4" t="n">
-        <v>-71.0534</v>
+        <v>-71.053</v>
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
-          <t>Cheveux gris, veston marine</t>
+          <t>Manches relevées, stylo rouge</t>
         </is>
       </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
-          <t>Complet, épinglette de ville</t>
+          <t>Chemise de rédaction</t>
         </is>
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>Poignée de main</t>
+          <t>Stylo rouge</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>portraits/121-gilles-dufour-web.webp</t>
+          <t>portraits/134-francois-cote-web.webp</t>
         </is>
       </c>
       <c r="N164" s="2" t="inlineStr">
         <is>
-          <t>Dufour</t>
+          <t>Côté</t>
         </is>
       </c>
       <c r="O164" s="2" t="inlineStr">
         <is>
-          <t>hôtel de ville</t>
+          <t>presse</t>
         </is>
       </c>
       <c r="P164" s="2" t="inlineStr">
         <is>
-          <t>Fils d’Albert Dufour — maire de Saguenay</t>
+          <t>Patron d’Olivier Savard — ex-patron de JP</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
         <is>
-          <t>Hélène Samson</t>
-        </is>
-      </c>
-      <c r="B165" s="5" t="n"/>
+          <t>Gaétan Bossé</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Le Bouquiniste</t>
+        </is>
+      </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D165" s="6" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>Retraitée — ex-secrétaire de palais</t>
+          <t>Bouquiniste — livres usagés</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
@@ -12371,65 +12375,69 @@
       </c>
       <c r="G165" s="5" t="inlineStr">
         <is>
-          <t>149, Rue Bégin</t>
+          <t>312, Rue Bossé</t>
         </is>
       </c>
       <c r="H165" s="7" t="n">
-        <v>48.4213</v>
+        <v>48.42445</v>
       </c>
       <c r="I165" s="7" t="n">
-        <v>-71.0574</v>
+        <v>-71.07605</v>
       </c>
       <c r="J165" s="5" t="inlineStr">
         <is>
-          <t>Cheveux soignés, manteau beige</t>
+          <t>Barbe grise, lunettes sur le front</t>
         </is>
       </c>
       <c r="K165" s="5" t="inlineStr">
         <is>
-          <t>Manteau beige</t>
+          <t>Veste de laine sur chemise à carreaux</t>
         </is>
       </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
-          <t>Sac à main</t>
+          <t>Livre relié sous le bras</t>
         </is>
       </c>
       <c r="M165" s="5" t="inlineStr">
         <is>
-          <t>portraits/168-helene-samson-web.webp</t>
+          <t>portraits/184-gaetan-bosse-web.webp</t>
         </is>
       </c>
       <c r="N165" s="5" t="inlineStr">
         <is>
-          <t>Samson</t>
+          <t>Bossé</t>
         </is>
       </c>
       <c r="O165" s="5" t="n"/>
       <c r="P165" s="5" t="inlineStr">
         <is>
-          <t>Mère de Pierre Samson</t>
+          <t>Frère de Stéphane Bossé</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Isabelle Gagné</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="n"/>
+          <t>Gilles Dufour</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Monsieur le Maire</t>
+        </is>
+      </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D166" s="3" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>Députée — Assemblée nationale</t>
+          <t>Maire de Saguenay</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -12439,73 +12447,69 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>145, Rue Racine Est</t>
+          <t>201, Rue Racine Est</t>
         </is>
       </c>
       <c r="H166" s="4" t="n">
-        <v>48.4279</v>
+        <v>48.4282</v>
       </c>
       <c r="I166" s="4" t="n">
-        <v>-71.0531</v>
+        <v>-71.0534</v>
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
-          <t>Carré blond, blazer rouge</t>
+          <t>Cheveux gris, veston marine</t>
         </is>
       </c>
       <c r="K166" s="2" t="inlineStr">
         <is>
-          <t>Blazer rouge</t>
+          <t>Complet, épinglette de ville</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>Épinglette fleurdelisé</t>
+          <t>Poignée de main</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr">
         <is>
-          <t>portraits/122-isabelle-gagne-web.webp</t>
+          <t>portraits/121-gilles-dufour-web.webp</t>
         </is>
       </c>
       <c r="N166" s="2" t="inlineStr">
         <is>
-          <t>Gagné</t>
+          <t>Dufour</t>
         </is>
       </c>
       <c r="O166" s="2" t="inlineStr">
         <is>
-          <t>politique</t>
+          <t>hôtel de ville</t>
         </is>
       </c>
       <c r="P166" s="2" t="inlineStr">
         <is>
-          <t>Célibataire</t>
+          <t>Fils d’Albert Dufour — maire de Saguenay</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>Jonathan Roy</t>
-        </is>
-      </c>
-      <c r="B167" s="5" t="inlineStr">
-        <is>
-          <t>Johnny Fake</t>
-        </is>
-      </c>
+          <t>Hélène Samson</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="n"/>
       <c r="C167" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D167" s="6" t="n">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>Arnaqueur — fausses identités</t>
+          <t>Retraitée — ex-secrétaire de palais</t>
         </is>
       </c>
       <c r="F167" s="5" t="inlineStr">
@@ -12515,73 +12519,65 @@
       </c>
       <c r="G167" s="5" t="inlineStr">
         <is>
-          <t>1186, Boulevard Talbot</t>
+          <t>149, Rue Bégin</t>
         </is>
       </c>
       <c r="H167" s="7" t="n">
-        <v>48.3986</v>
+        <v>48.4213</v>
       </c>
       <c r="I167" s="7" t="n">
-        <v>-71.0675</v>
+        <v>-71.0574</v>
       </c>
       <c r="J167" s="5" t="inlineStr">
         <is>
-          <t>Cheveux gominés, sourire</t>
+          <t>Cheveux soignés, manteau beige</t>
         </is>
       </c>
       <c r="K167" s="5" t="inlineStr">
         <is>
-          <t>Complet cheap</t>
+          <t>Manteau beige</t>
         </is>
       </c>
       <c r="L167" s="5" t="inlineStr">
         <is>
-          <t>Trois cellulaires</t>
+          <t>Sac à main</t>
         </is>
       </c>
       <c r="M167" s="5" t="inlineStr">
         <is>
-          <t>portraits/119-jonathan-roy-web.webp</t>
+          <t>portraits/168-helene-samson-web.webp</t>
         </is>
       </c>
       <c r="N167" s="5" t="inlineStr">
         <is>
-          <t>Roy</t>
-        </is>
-      </c>
-      <c r="O167" s="5" t="inlineStr">
-        <is>
-          <t>arnaque</t>
-        </is>
-      </c>
+          <t>Samson</t>
+        </is>
+      </c>
+      <c r="O167" s="5" t="n"/>
       <c r="P167" s="5" t="inlineStr">
         <is>
-          <t>Célibataire — croise Alex Tremblay</t>
+          <t>Mère de Pierre Samson</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Julien Gagné</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>Le Volant</t>
-        </is>
-      </c>
+          <t>Isabelle Gagné</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="n"/>
       <c r="C168" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D168" s="3" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Chauffeur de voiture de ville</t>
+          <t>Députée — Assemblée nationale</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -12591,56 +12587,60 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>1188, Boulevard Talbot</t>
+          <t>145, Rue Racine Est</t>
         </is>
       </c>
       <c r="H168" s="4" t="n">
-        <v>48.3983</v>
+        <v>48.4279</v>
       </c>
       <c r="I168" s="4" t="n">
-        <v>-71.06780000000001</v>
+        <v>-71.0531</v>
       </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
-          <t>Complet noir, oreillette</t>
+          <t>Carré blond, blazer rouge</t>
         </is>
       </c>
       <c r="K168" s="2" t="inlineStr">
         <is>
-          <t>Complet noir</t>
+          <t>Blazer rouge</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>VUS noir</t>
+          <t>Épinglette fleurdelisé</t>
         </is>
       </c>
       <c r="M168" s="2" t="inlineStr">
         <is>
-          <t>portraits/157-julien-gagne-web.webp</t>
+          <t>portraits/122-isabelle-gagne-web.webp</t>
         </is>
       </c>
       <c r="N168" s="2" t="inlineStr">
         <is>
-          <t>Santini</t>
-        </is>
-      </c>
-      <c r="O168" s="2" t="n"/>
+          <t>Gagné</t>
+        </is>
+      </c>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>politique</t>
+        </is>
+      </c>
       <c r="P168" s="2" t="inlineStr">
         <is>
-          <t>Chauffeur de Vittorio</t>
+          <t>Célibataire</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="inlineStr">
         <is>
-          <t>Justin Chen</t>
+          <t>Jonathan Roy</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
         <is>
-          <t>Junior Talbot</t>
+          <t>Johnny Fake</t>
         </is>
       </c>
       <c r="C169" s="6" t="inlineStr">
@@ -12649,11 +12649,11 @@
         </is>
       </c>
       <c r="D169" s="6" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>Étudiant en administration (Cégep de Chicoutimi)</t>
+          <t>Arnaqueur — fausses identités</t>
         </is>
       </c>
       <c r="F169" s="5" t="inlineStr">
@@ -12663,56 +12663,60 @@
       </c>
       <c r="G169" s="5" t="inlineStr">
         <is>
-          <t>1180, Boulevard Talbot</t>
+          <t>1186, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H169" s="7" t="n">
-        <v>48.398223</v>
+        <v>48.3986</v>
       </c>
       <c r="I169" s="7" t="n">
-        <v>-71.06763599999999</v>
+        <v>-71.0675</v>
       </c>
       <c r="J169" s="5" t="inlineStr">
         <is>
-          <t>Métis, Moncler propre</t>
+          <t>Cheveux gominés, sourire</t>
         </is>
       </c>
       <c r="K169" s="5" t="inlineStr">
         <is>
-          <t>Moncler noir</t>
+          <t>Complet cheap</t>
         </is>
       </c>
       <c r="L169" s="5" t="inlineStr">
         <is>
-          <t>Paye trop cher</t>
+          <t>Trois cellulaires</t>
         </is>
       </c>
       <c r="M169" s="5" t="inlineStr">
         <is>
-          <t>portraits/26-justin-chen-web.webp</t>
+          <t>portraits/119-jonathan-roy-web.webp</t>
         </is>
       </c>
       <c r="N169" s="5" t="inlineStr">
         <is>
-          <t>Chen</t>
-        </is>
-      </c>
-      <c r="O169" s="5" t="n"/>
+          <t>Roy</t>
+        </is>
+      </c>
+      <c r="O169" s="5" t="inlineStr">
+        <is>
+          <t>arnaque</t>
+        </is>
+      </c>
       <c r="P169" s="5" t="inlineStr">
         <is>
-          <t>Fils de Mei</t>
+          <t>Célibataire — croise Alex Tremblay</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Jérémie Côté</t>
+          <t>Julien Gagné</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Ti-Poste</t>
+          <t>Le Volant</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -12721,11 +12725,11 @@
         </is>
       </c>
       <c r="D170" s="3" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>Facteur — Postes Canada</t>
+          <t>Chauffeur de voiture de ville</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -12735,69 +12739,69 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>145, Rue Sainte-Anne</t>
+          <t>1188, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H170" s="4" t="n">
-        <v>48.42915</v>
+        <v>48.3983</v>
       </c>
       <c r="I170" s="4" t="n">
-        <v>-71.06835</v>
+        <v>-71.06780000000001</v>
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>Barbe taillée, joues rouges</t>
+          <t>Complet noir, oreillette</t>
         </is>
       </c>
       <c r="K170" s="2" t="inlineStr">
         <is>
-          <t>Parka de facteur à bandes</t>
+          <t>Complet noir</t>
         </is>
       </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
-          <t>Sacoche de courrier</t>
+          <t>VUS noir</t>
         </is>
       </c>
       <c r="M170" s="2" t="inlineStr">
         <is>
-          <t>portraits/187-jeremie-cote-web.webp</t>
+          <t>portraits/157-julien-gagne-web.webp</t>
         </is>
       </c>
       <c r="N170" s="2" t="inlineStr">
         <is>
-          <t>Côté</t>
-        </is>
-      </c>
-      <c r="O170" s="2" t="inlineStr">
-        <is>
-          <t>poste</t>
-        </is>
-      </c>
+          <t>Santini</t>
+        </is>
+      </c>
+      <c r="O170" s="2" t="n"/>
       <c r="P170" s="2" t="inlineStr">
         <is>
-          <t>Neveu d’Alain Côté</t>
+          <t>Chauffeur de Vittorio</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="inlineStr">
         <is>
-          <t>Laurie Lavoie</t>
-        </is>
-      </c>
-      <c r="B171" s="5" t="n"/>
+          <t>Justin Chen</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Junior Talbot</t>
+        </is>
+      </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D171" s="6" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>Étudiante en psychologie (UQAC)</t>
+          <t>Étudiant en administration (Cégep de Chicoutimi)</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
@@ -12807,69 +12811,69 @@
       </c>
       <c r="G171" s="5" t="inlineStr">
         <is>
-          <t>555, Boulevard de l'Université</t>
+          <t>1180, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H171" s="7" t="n">
-        <v>48.421623</v>
+        <v>48.398223</v>
       </c>
       <c r="I171" s="7" t="n">
-        <v>-71.07566199999999</v>
+        <v>-71.06763599999999</v>
       </c>
       <c r="J171" s="5" t="inlineStr">
         <is>
-          <t>Cheveux longs châtains, hoodie UQAC</t>
+          <t>Métis, Moncler propre</t>
         </is>
       </c>
       <c r="K171" s="5" t="inlineStr">
         <is>
-          <t>Hoodie UQAC</t>
+          <t>Moncler noir</t>
         </is>
       </c>
       <c r="L171" s="5" t="inlineStr">
         <is>
-          <t>Livre psycho</t>
+          <t>Paye trop cher</t>
         </is>
       </c>
       <c r="M171" s="5" t="inlineStr">
         <is>
-          <t>portraits/36-laurie-lavoie-web.webp</t>
+          <t>portraits/26-justin-chen-web.webp</t>
         </is>
       </c>
       <c r="N171" s="5" t="inlineStr">
         <is>
-          <t>Lavoie</t>
-        </is>
-      </c>
-      <c r="O171" s="5" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="O171" s="5" t="n"/>
       <c r="P171" s="5" t="inlineStr">
         <is>
-          <t>Sœur de JP</t>
+          <t>Fils de Mei</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Lise Gauthier</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="n"/>
+          <t>Jérémie Côté</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Ti-Poste</t>
+        </is>
+      </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D172" s="3" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>Infirmière clinicienne — CLSC</t>
+          <t>Facteur — Postes Canada</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
@@ -12879,51 +12883,55 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>222, Rue du Havre</t>
+          <t>145, Rue Sainte-Anne</t>
         </is>
       </c>
       <c r="H172" s="4" t="n">
-        <v>48.4293</v>
+        <v>48.42915</v>
       </c>
       <c r="I172" s="4" t="n">
-        <v>-71.05445</v>
+        <v>-71.06835</v>
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>Cheveux blancs courts, lunettes à chaînette</t>
+          <t>Barbe taillée, joues rouges</t>
         </is>
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>Cardigan bourgogne sur uniforme</t>
+          <t>Parka de facteur à bandes</t>
         </is>
       </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
-          <t>Tensiomètre</t>
+          <t>Sacoche de courrier</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr">
         <is>
-          <t>portraits/188-lise-gauthier-web.webp</t>
+          <t>portraits/187-jeremie-cote-web.webp</t>
         </is>
       </c>
       <c r="N172" s="2" t="inlineStr">
         <is>
-          <t>Gauthier</t>
-        </is>
-      </c>
-      <c r="O172" s="2" t="n"/>
+          <t>Côté</t>
+        </is>
+      </c>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>poste</t>
+        </is>
+      </c>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>Tante de Steve et Chantal Gauthier</t>
+          <t>Neveu d’Alain Côté</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="inlineStr">
         <is>
-          <t>Louise Villeneuve</t>
+          <t>Laurie Lavoie</t>
         </is>
       </c>
       <c r="B173" s="5" t="n"/>
@@ -12933,11 +12941,11 @@
         </is>
       </c>
       <c r="D173" s="6" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>Juge — Cour du Québec</t>
+          <t>Étudiante en psychologie (UQAC)</t>
         </is>
       </c>
       <c r="F173" s="5" t="inlineStr">
@@ -12947,73 +12955,69 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>227, Rue Racine Est</t>
+          <t>555, Boulevard de l'Université</t>
         </is>
       </c>
       <c r="H173" s="7" t="n">
-        <v>48.4275</v>
+        <v>48.421623</v>
       </c>
       <c r="I173" s="7" t="n">
-        <v>-71.05419999999999</v>
+        <v>-71.07566199999999</v>
       </c>
       <c r="J173" s="5" t="inlineStr">
         <is>
-          <t>Regard sévère, toge</t>
+          <t>Cheveux longs châtains, hoodie UQAC</t>
         </is>
       </c>
       <c r="K173" s="5" t="inlineStr">
         <is>
-          <t>Toge</t>
+          <t>Hoodie UQAC</t>
         </is>
       </c>
       <c r="L173" s="5" t="inlineStr">
         <is>
-          <t>Marteau de bois</t>
+          <t>Livre psycho</t>
         </is>
       </c>
       <c r="M173" s="5" t="inlineStr">
         <is>
-          <t>portraits/127-louise-villeneuve-web.webp</t>
+          <t>portraits/36-laurie-lavoie-web.webp</t>
         </is>
       </c>
       <c r="N173" s="5" t="inlineStr">
         <is>
-          <t>Villeneuve</t>
+          <t>Lavoie</t>
         </is>
       </c>
       <c r="O173" s="5" t="inlineStr">
         <is>
-          <t>palais</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="P173" s="5" t="inlineStr">
         <is>
-          <t>Collègue de Catherine Samson</t>
+          <t>Sœur de JP</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Maria Santini</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>Donna Maria</t>
-        </is>
-      </c>
+          <t>Lise Gauthier</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="n"/>
       <c r="C174" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D174" s="3" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>Matriarche — restaurant familial</t>
+          <t>Infirmière clinicienne — CLSC</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
@@ -13023,69 +13027,65 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>200, Rue Racine Est</t>
+          <t>222, Rue du Havre</t>
         </is>
       </c>
       <c r="H174" s="4" t="n">
-        <v>48.42815</v>
+        <v>48.4293</v>
       </c>
       <c r="I174" s="4" t="n">
-        <v>-71.0543</v>
+        <v>-71.05445</v>
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>Cheveux sombres, perles</t>
+          <t>Cheveux blancs courts, lunettes à chaînette</t>
         </is>
       </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
-          <t>Robe noire</t>
+          <t>Cardigan bourgogne sur uniforme</t>
         </is>
       </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
-          <t>Rosaire au poignet</t>
+          <t>Tensiomètre</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr">
         <is>
-          <t>portraits/152-maria-santini-web.webp</t>
+          <t>portraits/188-lise-gauthier-web.webp</t>
         </is>
       </c>
       <c r="N174" s="2" t="inlineStr">
         <is>
-          <t>Santini</t>
+          <t>Gauthier</t>
         </is>
       </c>
       <c r="O174" s="2" t="n"/>
       <c r="P174" s="2" t="inlineStr">
         <is>
-          <t>Épouse de Vittorio</t>
+          <t>Tante de Steve et Chantal Gauthier</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="inlineStr">
         <is>
-          <t>Marie-Ève Boucher</t>
-        </is>
-      </c>
-      <c r="B175" s="5" t="inlineStr">
-        <is>
-          <t>La Plume</t>
-        </is>
-      </c>
+          <t>Louise Villeneuve</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="n"/>
       <c r="C175" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D175" s="6" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>Journaliste — quotidien régional</t>
+          <t>Juge — Cour du Québec</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
@@ -13095,65 +13095,73 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>412, Rue Jacques-Cartier Ouest</t>
+          <t>227, Rue Racine Est</t>
         </is>
       </c>
       <c r="H175" s="7" t="n">
-        <v>48.4268</v>
+        <v>48.4275</v>
       </c>
       <c r="I175" s="7" t="n">
-        <v>-71.0699</v>
+        <v>-71.05419999999999</v>
       </c>
       <c r="J175" s="5" t="inlineStr">
         <is>
-          <t>Cheveux courts noirs, regard vif</t>
+          <t>Regard sévère, toge</t>
         </is>
       </c>
       <c r="K175" s="5" t="inlineStr">
         <is>
-          <t>Trench, cordon de presse</t>
+          <t>Toge</t>
         </is>
       </c>
       <c r="L175" s="5" t="inlineStr">
         <is>
-          <t>Calepin et téléphone</t>
+          <t>Marteau de bois</t>
         </is>
       </c>
       <c r="M175" s="5" t="inlineStr">
         <is>
-          <t>portraits/185-marie-eve-boucher-web.webp</t>
+          <t>portraits/127-louise-villeneuve-web.webp</t>
         </is>
       </c>
       <c r="N175" s="5" t="inlineStr">
         <is>
-          <t>Bossé</t>
-        </is>
-      </c>
-      <c r="O175" s="5" t="n"/>
+          <t>Villeneuve</t>
+        </is>
+      </c>
+      <c r="O175" s="5" t="inlineStr">
+        <is>
+          <t>palais</t>
+        </is>
+      </c>
       <c r="P175" s="5" t="inlineStr">
         <is>
-          <t>Conjointe de Stéphane Bossé — cousine de Normand Boucher</t>
+          <t>Collègue de Catherine Samson</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Mei Chen</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="n"/>
+          <t>Lucien Gagné</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Le Proprio des étudiants</t>
+        </is>
+      </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D176" s="3" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>Préposée d’hôtel</t>
+          <t>Propriétaire — logements étudiants</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
@@ -13163,56 +13171,60 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>1182, Boulevard Talbot</t>
+          <t>320, Rue Saint-Vallier</t>
         </is>
       </c>
       <c r="H176" s="4" t="n">
-        <v>48.39835</v>
+        <v>48.42645</v>
       </c>
       <c r="I176" s="4" t="n">
-        <v>-71.06775</v>
+        <v>-71.0502</v>
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>Chinoise, chignon, calme</t>
+          <t>Chauve, lunettes sur le nez</t>
         </is>
       </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
-          <t>Uniforme hôtel</t>
+          <t>Veste matelassée sur chemise à carreaux</t>
         </is>
       </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
-          <t>Badges de chambre</t>
+          <t>Trousseau de clés</t>
         </is>
       </c>
       <c r="M176" s="2" t="inlineStr">
         <is>
-          <t>portraits/63-mei-chen-web.webp</t>
+          <t>portraits/210-lucien-gagne-web.webp</t>
         </is>
       </c>
       <c r="N176" s="2" t="inlineStr">
         <is>
-          <t>Chen</t>
-        </is>
-      </c>
-      <c r="O176" s="2" t="n"/>
+          <t>Gagné</t>
+        </is>
+      </c>
+      <c r="O176" s="2" t="inlineStr">
+        <is>
+          <t>logements</t>
+        </is>
+      </c>
       <c r="P176" s="2" t="inlineStr">
         <is>
-          <t>Mère de Justin Chen</t>
+          <t>Oncle d’Isabelle Gagné — propriétaire d’Emma, Moussa et William</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="inlineStr">
         <is>
-          <t>Mgr Paul Tremblay</t>
+          <t>Maria Santini</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
         <is>
-          <t>Monseigneur</t>
+          <t>Donna Maria</t>
         </is>
       </c>
       <c r="C177" s="6" t="inlineStr">
@@ -13221,11 +13233,11 @@
         </is>
       </c>
       <c r="D177" s="6" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E177" s="5" t="inlineStr">
         <is>
-          <t>Évêque — diocèse de Chicoutimi</t>
+          <t>Matriarche — restaurant familial</t>
         </is>
       </c>
       <c r="F177" s="5" t="inlineStr">
@@ -13235,60 +13247,56 @@
       </c>
       <c r="G177" s="5" t="inlineStr">
         <is>
-          <t>602, Rue Racine Est</t>
+          <t>200, Rue Racine Est</t>
         </is>
       </c>
       <c r="H177" s="7" t="n">
-        <v>48.4268</v>
+        <v>48.42815</v>
       </c>
       <c r="I177" s="7" t="n">
-        <v>-71.0538</v>
+        <v>-71.0543</v>
       </c>
       <c r="J177" s="5" t="inlineStr">
         <is>
-          <t>Cheveux blancs, col romain</t>
+          <t>Cheveux sombres, perles</t>
         </is>
       </c>
       <c r="K177" s="5" t="inlineStr">
         <is>
-          <t>Soutane, rabat violet</t>
+          <t>Robe noire</t>
         </is>
       </c>
       <c r="L177" s="5" t="inlineStr">
         <is>
-          <t>Anneau pastoral</t>
+          <t>Rosaire au poignet</t>
         </is>
       </c>
       <c r="M177" s="5" t="inlineStr">
         <is>
-          <t>portraits/126-mgr-paul-tremblay-web.webp</t>
+          <t>portraits/152-maria-santini-web.webp</t>
         </is>
       </c>
       <c r="N177" s="5" t="inlineStr">
         <is>
-          <t>Tremblay</t>
-        </is>
-      </c>
-      <c r="O177" s="5" t="inlineStr">
-        <is>
-          <t>Église</t>
-        </is>
-      </c>
+          <t>Santini</t>
+        </is>
+      </c>
+      <c r="O177" s="5" t="n"/>
       <c r="P177" s="5" t="inlineStr">
         <is>
-          <t>Supérieur de Lucien Lacroix</t>
+          <t>Épouse de Vittorio</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Nico Santini</t>
+          <t>Marie-Ève Boucher</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Nico</t>
+          <t>La Plume</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
@@ -13297,11 +13305,11 @@
         </is>
       </c>
       <c r="D178" s="3" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>Préposé à la sécurité — restaurant</t>
+          <t>Journaliste — quotidien régional</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
@@ -13311,51 +13319,51 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>202, Rue Racine Est</t>
+          <t>412, Rue Jacques-Cartier Ouest</t>
         </is>
       </c>
       <c r="H178" s="4" t="n">
-        <v>48.4282</v>
+        <v>48.4268</v>
       </c>
       <c r="I178" s="4" t="n">
-        <v>-71.05459999999999</v>
+        <v>-71.0699</v>
       </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>Cheveux gominés, veste cuir</t>
+          <t>Cheveux courts noirs, regard vif</t>
         </is>
       </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
-          <t>Veste de cuir</t>
+          <t>Trench, cordon de presse</t>
         </is>
       </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
-          <t>Sourire de défi</t>
+          <t>Calepin et téléphone</t>
         </is>
       </c>
       <c r="M178" s="2" t="inlineStr">
         <is>
-          <t>portraits/160-nico-santini-web.webp</t>
+          <t>portraits/185-marie-eve-boucher-web.webp</t>
         </is>
       </c>
       <c r="N178" s="2" t="inlineStr">
         <is>
-          <t>Santini</t>
+          <t>Bossé</t>
         </is>
       </c>
       <c r="O178" s="2" t="n"/>
       <c r="P178" s="2" t="inlineStr">
         <is>
-          <t>Fils de Vittorio et Maria</t>
+          <t>Conjointe de Stéphane Bossé — cousine de Normand Boucher</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="inlineStr">
         <is>
-          <t>Olivier Savard</t>
+          <t>Maïka Gauthier</t>
         </is>
       </c>
       <c r="B179" s="5" t="n"/>
@@ -13365,11 +13373,11 @@
         </is>
       </c>
       <c r="D179" s="6" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>Journaliste — Le Quotidien</t>
+          <t>Étudiante en soins infirmiers (Cégep de Chicoutimi) — caissière de pharmacie</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
@@ -13379,69 +13387,65 @@
       </c>
       <c r="G179" s="5" t="inlineStr">
         <is>
-          <t>100, Rue Racine Est</t>
+          <t>152, Rue LaFontaine</t>
         </is>
       </c>
       <c r="H179" s="7" t="n">
-        <v>48.4278</v>
+        <v>48.4205</v>
       </c>
       <c r="I179" s="7" t="n">
-        <v>-71.05289999999999</v>
+        <v>-71.06075</v>
       </c>
       <c r="J179" s="5" t="inlineStr">
         <is>
-          <t>Barbe, sacoche</t>
+          <t>Queue de cheval châtaine, sourire poli</t>
         </is>
       </c>
       <c r="K179" s="5" t="inlineStr">
         <is>
-          <t>Manteau de ville</t>
+          <t>Sarrau blanc de pharmacie</t>
         </is>
       </c>
       <c r="L179" s="5" t="inlineStr">
         <is>
-          <t>Carnet spiralé</t>
+          <t>Étiquette de nom</t>
         </is>
       </c>
       <c r="M179" s="5" t="inlineStr">
         <is>
-          <t>portraits/78-olivier-savard-web.webp</t>
+          <t>portraits/207-maika-gauthier-web.webp</t>
         </is>
       </c>
       <c r="N179" s="5" t="inlineStr">
         <is>
-          <t>Savard</t>
+          <t>Gauthier</t>
         </is>
       </c>
       <c r="O179" s="5" t="n"/>
       <c r="P179" s="5" t="inlineStr">
         <is>
-          <t>Célibataire — ex-collègue de JP</t>
+          <t>Nièce de Lise Gauthier — cousine de Steve et Chantal</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Patrick Lapointe</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>Pat</t>
-        </is>
-      </c>
+          <t>Mei Chen</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="n"/>
       <c r="C180" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D180" s="3" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneur en construction</t>
+          <t>Préposée d’hôtel</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -13451,60 +13455,56 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>1250, Boulevard Talbot</t>
+          <t>1182, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H180" s="4" t="n">
-        <v>48.3985</v>
+        <v>48.39835</v>
       </c>
       <c r="I180" s="4" t="n">
-        <v>-71.06276</v>
+        <v>-71.06775</v>
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>Polo construction</t>
+          <t>Chinoise, chignon, calme</t>
         </is>
       </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
-          <t>Polo construction</t>
+          <t>Uniforme hôtel</t>
         </is>
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>Devis 400k</t>
+          <t>Badges de chambre</t>
         </is>
       </c>
       <c r="M180" s="2" t="inlineStr">
         <is>
-          <t>portraits/39-patrick-lapointe-web.webp</t>
+          <t>portraits/63-mei-chen-web.webp</t>
         </is>
       </c>
       <c r="N180" s="2" t="inlineStr">
         <is>
-          <t>Lapointe</t>
-        </is>
-      </c>
-      <c r="O180" s="2" t="inlineStr">
-        <is>
-          <t>Marco</t>
-        </is>
-      </c>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="O180" s="2" t="n"/>
       <c r="P180" s="2" t="inlineStr">
         <is>
-          <t>Frère de Marco</t>
+          <t>Mère de Justin Chen</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="inlineStr">
         <is>
-          <t>Paul-André Côté</t>
+          <t>Mgr Paul Tremblay</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
         <is>
-          <t>Le Chiffre</t>
+          <t>Monseigneur</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
@@ -13513,11 +13513,11 @@
         </is>
       </c>
       <c r="D181" s="6" t="n">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>Comptable — sociétés-écrans</t>
+          <t>Évêque — diocèse de Chicoutimi</t>
         </is>
       </c>
       <c r="F181" s="5" t="inlineStr">
@@ -13527,69 +13527,69 @@
       </c>
       <c r="G181" s="5" t="inlineStr">
         <is>
-          <t>1252, Boulevard Talbot</t>
+          <t>602, Rue Racine Est</t>
         </is>
       </c>
       <c r="H181" s="7" t="n">
-        <v>48.39855</v>
+        <v>48.4268</v>
       </c>
       <c r="I181" s="7" t="n">
-        <v>-71.0629</v>
+        <v>-71.0538</v>
       </c>
       <c r="J181" s="5" t="inlineStr">
         <is>
-          <t>Maigre, lunettes cheap</t>
+          <t>Cheveux blancs, col romain</t>
         </is>
       </c>
       <c r="K181" s="5" t="inlineStr">
         <is>
-          <t>Chemise et classeur</t>
+          <t>Soutane, rabat violet</t>
         </is>
       </c>
       <c r="L181" s="5" t="inlineStr">
         <is>
-          <t>Tableurs</t>
+          <t>Anneau pastoral</t>
         </is>
       </c>
       <c r="M181" s="5" t="inlineStr">
         <is>
-          <t>portraits/156-paul-andre-cote-web.webp</t>
+          <t>portraits/126-mgr-paul-tremblay-web.webp</t>
         </is>
       </c>
       <c r="N181" s="5" t="inlineStr">
         <is>
-          <t>Santini</t>
-        </is>
-      </c>
-      <c r="O181" s="5" t="n"/>
+          <t>Tremblay</t>
+        </is>
+      </c>
+      <c r="O181" s="5" t="inlineStr">
+        <is>
+          <t>Église</t>
+        </is>
+      </c>
       <c r="P181" s="5" t="inlineStr">
         <is>
-          <t>Comptable du clan — croise Bertrand Gagnon</t>
+          <t>Supérieur de Lucien Lacroix</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Pierre Samson</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>L'Enquêteur</t>
-        </is>
-      </c>
+          <t>Moussa Diallo</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="n"/>
       <c r="C182" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D182" s="3" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>Policier — Service de police de Saguenay, stupéfiants</t>
+          <t>Étudiant en informatique (UQAC)</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -13599,56 +13599,56 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>145, Rue Bégin</t>
+          <t>318, Rue Saint-Vallier</t>
         </is>
       </c>
       <c r="H182" s="4" t="n">
-        <v>48.421205</v>
+        <v>48.4264</v>
       </c>
       <c r="I182" s="4" t="n">
-        <v>-71.057355</v>
+        <v>-71.05025000000001</v>
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>Cernes violacés</t>
+          <t>Grand, sourire large</t>
         </is>
       </c>
       <c r="K182" s="2" t="inlineStr">
         <is>
-          <t>Pardessus brun-beige</t>
+          <t>Doudoune sur hoodie</t>
         </is>
       </c>
       <c r="L182" s="2" t="inlineStr">
         <is>
-          <t>Clique Bic bleu</t>
+          <t>Écouteurs autour du cou</t>
         </is>
       </c>
       <c r="M182" s="2" t="inlineStr">
         <is>
-          <t>portraits/07-pierre-samson-web.webp</t>
+          <t>portraits/205-moussa-diallo-web.webp</t>
         </is>
       </c>
       <c r="N182" s="2" t="inlineStr">
         <is>
-          <t>Samson</t>
+          <t>Diallo</t>
         </is>
       </c>
       <c r="O182" s="2" t="n"/>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>Fils d’Hélène Samson — époux de Catherine</t>
+          <t>Célibataire — colocataire d’Emma Boucher et William Lavoie</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="inlineStr">
         <is>
-          <t>Sofia Santini</t>
+          <t>Nico Santini</t>
         </is>
       </c>
       <c r="B183" s="5" t="inlineStr">
         <is>
-          <t>Sofi</t>
+          <t>Nico</t>
         </is>
       </c>
       <c r="C183" s="6" t="inlineStr">
@@ -13657,11 +13657,11 @@
         </is>
       </c>
       <c r="D183" s="6" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>Élève du secondaire — aide au restaurant familial</t>
+          <t>Préposé à la sécurité — restaurant</t>
         </is>
       </c>
       <c r="F183" s="5" t="inlineStr">
@@ -13671,33 +13671,33 @@
       </c>
       <c r="G183" s="5" t="inlineStr">
         <is>
-          <t>204, Rue Racine Est</t>
+          <t>202, Rue Racine Est</t>
         </is>
       </c>
       <c r="H183" s="7" t="n">
-        <v>48.42825</v>
+        <v>48.4282</v>
       </c>
       <c r="I183" s="7" t="n">
-        <v>-71.05475</v>
+        <v>-71.05459999999999</v>
       </c>
       <c r="J183" s="5" t="inlineStr">
         <is>
-          <t>Cheveux noirs ondulés, sourire en coin</t>
+          <t>Cheveux gominés, veste cuir</t>
         </is>
       </c>
       <c r="K183" s="5" t="inlineStr">
         <is>
-          <t>Tablier noir de service</t>
+          <t>Veste de cuir</t>
         </is>
       </c>
       <c r="L183" s="5" t="inlineStr">
         <is>
-          <t>Cabaret à deux mains</t>
+          <t>Sourire de défi</t>
         </is>
       </c>
       <c r="M183" s="5" t="inlineStr">
         <is>
-          <t>portraits/177-sofia-santini-web.webp</t>
+          <t>portraits/160-nico-santini-web.webp</t>
         </is>
       </c>
       <c r="N183" s="5" t="inlineStr">
@@ -13708,28 +13708,32 @@
       <c r="O183" s="5" t="n"/>
       <c r="P183" s="5" t="inlineStr">
         <is>
-          <t>Fille de Nico Santini — petite-fille de Vittorio et Maria</t>
+          <t>Fils de Vittorio et Maria</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Sophie Labbé</t>
-        </is>
-      </c>
-      <c r="B184" s="2" t="n"/>
+          <t>Olivier Brassard</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Oli</t>
+        </is>
+      </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D184" s="3" t="n">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>Psychologue — clinique UQAC</t>
+          <t>Coursier à vélo — musicien</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -13739,69 +13743,65 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>555, Boulevard de l'Université</t>
+          <t>122, Rue Dréan</t>
         </is>
       </c>
       <c r="H184" s="4" t="n">
-        <v>48.4215</v>
+        <v>48.42615</v>
       </c>
       <c r="I184" s="4" t="n">
-        <v>-71.07550000000001</v>
+        <v>-71.08029999999999</v>
       </c>
       <c r="J184" s="2" t="inlineStr">
         <is>
-          <t>Chignon, lunettes</t>
+          <t>Moustache, casquette à l’envers</t>
         </is>
       </c>
       <c r="K184" s="2" t="inlineStr">
         <is>
-          <t>Cardigan</t>
+          <t>Veste en denim à écussons</t>
         </is>
       </c>
       <c r="L184" s="2" t="inlineStr">
         <is>
-          <t>Carnet de notes</t>
+          <t>Ukulélé sur le sac</t>
         </is>
       </c>
       <c r="M184" s="2" t="inlineStr">
         <is>
-          <t>portraits/104-sophie-labbe-web.webp</t>
+          <t>portraits/208-olivier-brassard-web.webp</t>
         </is>
       </c>
       <c r="N184" s="2" t="inlineStr">
         <is>
-          <t>Labbé</t>
+          <t>Brassard</t>
         </is>
       </c>
       <c r="O184" s="2" t="n"/>
       <c r="P184" s="2" t="inlineStr">
         <is>
-          <t>Célibataire — collègue de Laurie Lavoie</t>
+          <t>Neveu d’Émile Brassard</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="inlineStr">
         <is>
-          <t>Stéphane Bossé</t>
-        </is>
-      </c>
-      <c r="B185" s="5" t="inlineStr">
-        <is>
-          <t>Steph Patate</t>
-        </is>
-      </c>
+          <t>Olivier Savard</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="n"/>
       <c r="C185" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D185" s="6" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
-          <t>Cuisinier — casse-croûte</t>
+          <t>Journaliste — Le Quotidien</t>
         </is>
       </c>
       <c r="F185" s="5" t="inlineStr">
@@ -13811,65 +13811,69 @@
       </c>
       <c r="G185" s="5" t="inlineStr">
         <is>
-          <t>410, Rue Jacques-Cartier Ouest</t>
+          <t>100, Rue Racine Est</t>
         </is>
       </c>
       <c r="H185" s="7" t="n">
-        <v>48.42675</v>
+        <v>48.4278</v>
       </c>
       <c r="I185" s="7" t="n">
-        <v>-71.07004999999999</v>
+        <v>-71.05289999999999</v>
       </c>
       <c r="J185" s="5" t="inlineStr">
         <is>
-          <t>Cheveux ras, avant-bras tatoués</t>
+          <t>Barbe, sacoche</t>
         </is>
       </c>
       <c r="K185" s="5" t="inlineStr">
         <is>
-          <t>Tablier blanc taché</t>
+          <t>Manteau de ville</t>
         </is>
       </c>
       <c r="L185" s="5" t="inlineStr">
         <is>
-          <t>Spatule à la main</t>
+          <t>Carnet spiralé</t>
         </is>
       </c>
       <c r="M185" s="5" t="inlineStr">
         <is>
-          <t>portraits/186-stephane-bosse-web.webp</t>
+          <t>portraits/78-olivier-savard-web.webp</t>
         </is>
       </c>
       <c r="N185" s="5" t="inlineStr">
         <is>
-          <t>Bossé</t>
+          <t>Savard</t>
         </is>
       </c>
       <c r="O185" s="5" t="n"/>
       <c r="P185" s="5" t="inlineStr">
         <is>
-          <t>Frère de Gaétan Bossé — conjoint de Marie-Ève Boucher</t>
+          <t>Célibataire — ex-collègue de JP</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Valentina Rojas</t>
-        </is>
-      </c>
-      <c r="B186" s="2" t="n"/>
+          <t>Patrick Lapointe</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Pat</t>
+        </is>
+      </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D186" s="3" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>Épicière — produits latino-américains</t>
+          <t>Entrepreneur en construction</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
@@ -13879,56 +13883,60 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>318, Rue Bossé</t>
+          <t>1250, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H186" s="4" t="n">
-        <v>48.4245</v>
+        <v>48.3985</v>
       </c>
       <c r="I186" s="4" t="n">
-        <v>-71.07585</v>
+        <v>-71.06276</v>
       </c>
       <c r="J186" s="2" t="inlineStr">
         <is>
-          <t>Longs cheveux noirs, anneaux dorés</t>
+          <t>Polo construction</t>
         </is>
       </c>
       <c r="K186" s="2" t="inlineStr">
         <is>
-          <t>Tablier vert sur chandail</t>
+          <t>Polo construction</t>
         </is>
       </c>
       <c r="L186" s="2" t="inlineStr">
         <is>
-          <t>Caisse de plantains</t>
+          <t>Devis 400k</t>
         </is>
       </c>
       <c r="M186" s="2" t="inlineStr">
         <is>
-          <t>portraits/189-valentina-rojas-web.webp</t>
+          <t>portraits/39-patrick-lapointe-web.webp</t>
         </is>
       </c>
       <c r="N186" s="2" t="inlineStr">
         <is>
-          <t>Rojas</t>
-        </is>
-      </c>
-      <c r="O186" s="2" t="n"/>
+          <t>Lapointe</t>
+        </is>
+      </c>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
       <c r="P186" s="2" t="inlineStr">
         <is>
-          <t>Célibataire</t>
+          <t>Frère de Marco</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="inlineStr">
         <is>
-          <t>Vittorio Santini</t>
+          <t>Paul-André Côté</t>
         </is>
       </c>
       <c r="B187" s="5" t="inlineStr">
         <is>
-          <t>Don Vittorio</t>
+          <t>Le Chiffre</t>
         </is>
       </c>
       <c r="C187" s="6" t="inlineStr">
@@ -13937,11 +13945,11 @@
         </is>
       </c>
       <c r="D187" s="6" t="n">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
-          <t>Homme d’affaires — restauration et bars</t>
+          <t>Comptable — sociétés-écrans</t>
         </is>
       </c>
       <c r="F187" s="5" t="inlineStr">
@@ -13951,33 +13959,33 @@
       </c>
       <c r="G187" s="5" t="inlineStr">
         <is>
-          <t>200, Rue Racine Est</t>
+          <t>1252, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H187" s="7" t="n">
-        <v>48.4281</v>
+        <v>48.39855</v>
       </c>
       <c r="I187" s="7" t="n">
-        <v>-71.0545</v>
+        <v>-71.0629</v>
       </c>
       <c r="J187" s="5" t="inlineStr">
         <is>
-          <t>Cheveux argentés gominés, chevalière</t>
+          <t>Maigre, lunettes cheap</t>
         </is>
       </c>
       <c r="K187" s="5" t="inlineStr">
         <is>
-          <t>Manteau noir</t>
+          <t>Chemise et classeur</t>
         </is>
       </c>
       <c r="L187" s="5" t="inlineStr">
         <is>
-          <t>Chevalière en or</t>
+          <t>Tableurs</t>
         </is>
       </c>
       <c r="M187" s="5" t="inlineStr">
         <is>
-          <t>portraits/151-vittorio-santini-web.webp</t>
+          <t>portraits/156-paul-andre-cote-web.webp</t>
         </is>
       </c>
       <c r="N187" s="5" t="inlineStr">
@@ -13988,19 +13996,19 @@
       <c r="O187" s="5" t="n"/>
       <c r="P187" s="5" t="inlineStr">
         <is>
-          <t>Époux de Maria — tient Dévon à distance</t>
+          <t>Comptable du clan — croise Bertrand Gagnon</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Éric Simard</t>
+          <t>Pierre Samson</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Ti-Eric</t>
+          <t>L'Enquêteur</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -14009,11 +14017,11 @@
         </is>
       </c>
       <c r="D188" s="3" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>Étudiant — Cégep de Chicoutimi</t>
+          <t>Policier — Service de police de Saguenay, stupéfiants</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
@@ -14023,56 +14031,56 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>1184, Boulevard Talbot</t>
+          <t>145, Rue Bégin</t>
         </is>
       </c>
       <c r="H188" s="4" t="n">
-        <v>48.3984</v>
+        <v>48.421205</v>
       </c>
       <c r="I188" s="4" t="n">
-        <v>-71.06740000000001</v>
+        <v>-71.057355</v>
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>Casquette, jeans</t>
+          <t>Cernes violacés</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>Hoodie cégep</t>
+          <t>Pardessus brun-beige</t>
         </is>
       </c>
       <c r="L188" s="2" t="inlineStr">
         <is>
-          <t>Skateboard</t>
+          <t>Clique Bic bleu</t>
         </is>
       </c>
       <c r="M188" s="2" t="inlineStr">
         <is>
-          <t>portraits/100-eric-simard-web.webp</t>
+          <t>portraits/07-pierre-samson-web.webp</t>
         </is>
       </c>
       <c r="N188" s="2" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Samson</t>
         </is>
       </c>
       <c r="O188" s="2" t="n"/>
       <c r="P188" s="2" t="inlineStr">
         <is>
-          <t>Colocataire de Justin Chen</t>
+          <t>Fils d’Hélène Samson — époux de Catherine</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="5" t="inlineStr">
         <is>
-          <t>Antoine Lefèvre</t>
+          <t>Sofia Santini</t>
         </is>
       </c>
       <c r="B189" s="5" t="inlineStr">
         <is>
-          <t>Le Français</t>
+          <t>Sofi</t>
         </is>
       </c>
       <c r="C189" s="6" t="inlineStr">
@@ -14081,65 +14089,65 @@
         </is>
       </c>
       <c r="D189" s="6" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+          <t>Élève du secondaire — aide au restaurant familial</t>
         </is>
       </c>
       <c r="F189" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G189" s="5" t="inlineStr">
         <is>
-          <t>1125, Rue Saint-Dominique</t>
+          <t>204, Rue Racine Est</t>
         </is>
       </c>
       <c r="H189" s="7" t="n">
-        <v>48.421279</v>
+        <v>48.42825</v>
       </c>
       <c r="I189" s="7" t="n">
-        <v>-71.244586</v>
+        <v>-71.05475</v>
       </c>
       <c r="J189" s="5" t="inlineStr">
         <is>
-          <t>Barbe hipster</t>
+          <t>Cheveux noirs ondulés, sourire en coin</t>
         </is>
       </c>
       <c r="K189" s="5" t="inlineStr">
         <is>
-          <t>Friperie, caméra Sony</t>
+          <t>Tablier noir de service</t>
         </is>
       </c>
       <c r="L189" s="5" t="inlineStr">
         <is>
-          <t>Veut docu raw</t>
+          <t>Cabaret à deux mains</t>
         </is>
       </c>
       <c r="M189" s="5" t="inlineStr">
         <is>
-          <t>portraits/20-antoine-lefevre-web.webp</t>
+          <t>portraits/177-sofia-santini-web.webp</t>
         </is>
       </c>
       <c r="N189" s="5" t="inlineStr">
         <is>
-          <t>Lefèvre</t>
+          <t>Santini</t>
         </is>
       </c>
       <c r="O189" s="5" t="n"/>
       <c r="P189" s="5" t="inlineStr">
         <is>
-          <t>Frère de Camille</t>
+          <t>Fille de Nico Santini — petite-fille de Vittorio et Maria</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Audrey Lavoie</t>
+          <t>Sophie Labbé</t>
         </is>
       </c>
       <c r="B190" s="2" t="n"/>
@@ -14149,137 +14157,137 @@
         </is>
       </c>
       <c r="D190" s="3" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>Apprentie électricienne — aluminerie Rio Tinto Arvida</t>
+          <t>Psychologue — clinique UQAC</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>2135, Rue Davis</t>
+          <t>555, Boulevard de l'Université</t>
         </is>
       </c>
       <c r="H190" s="4" t="n">
-        <v>48.42455</v>
+        <v>48.4215</v>
       </c>
       <c r="I190" s="4" t="n">
-        <v>-71.18219999999999</v>
+        <v>-71.07550000000001</v>
       </c>
       <c r="J190" s="2" t="inlineStr">
         <is>
-          <t>Tresse blonde, lunettes de sécurité</t>
+          <t>Chignon, lunettes</t>
         </is>
       </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>Manteau orange haute visibilité</t>
+          <t>Cardigan</t>
         </is>
       </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
-          <t>Glacière à lunch</t>
+          <t>Carnet de notes</t>
         </is>
       </c>
       <c r="M190" s="2" t="inlineStr">
         <is>
-          <t>portraits/191-audrey-lavoie-web.webp</t>
+          <t>portraits/104-sophie-labbe-web.webp</t>
         </is>
       </c>
       <c r="N190" s="2" t="inlineStr">
         <is>
-          <t>Lavoie</t>
-        </is>
-      </c>
-      <c r="O190" s="2" t="inlineStr">
-        <is>
-          <t>Arvida</t>
-        </is>
-      </c>
+          <t>Labbé</t>
+        </is>
+      </c>
+      <c r="O190" s="2" t="n"/>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>Fille de Fernand Lavoie — collègue de Nicolas Gagné</t>
+          <t>Célibataire — collègue de Laurie Lavoie</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="5" t="inlineStr">
         <is>
-          <t>Benoit Larouche</t>
-        </is>
-      </c>
-      <c r="B191" s="5" t="n"/>
+          <t>Stéphane Bossé</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Steph Patate</t>
+        </is>
+      </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D191" s="6" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
-          <t>Enseignant — Cégep de Jonquière (ATM)</t>
+          <t>Cuisinier — casse-croûte</t>
         </is>
       </c>
       <c r="F191" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G191" s="5" t="inlineStr">
         <is>
-          <t>2505, Rue Saint-Hubert</t>
+          <t>410, Rue Jacques-Cartier Ouest</t>
         </is>
       </c>
       <c r="H191" s="7" t="n">
-        <v>48.416</v>
+        <v>48.42675</v>
       </c>
       <c r="I191" s="7" t="n">
-        <v>-71.253</v>
+        <v>-71.07004999999999</v>
       </c>
       <c r="J191" s="5" t="inlineStr">
         <is>
-          <t>Lunettes, barbe grise</t>
+          <t>Cheveux ras, avant-bras tatoués</t>
         </is>
       </c>
       <c r="K191" s="5" t="inlineStr">
         <is>
-          <t>Chemise et cardigan</t>
+          <t>Tablier blanc taché</t>
         </is>
       </c>
       <c r="L191" s="5" t="inlineStr">
         <is>
-          <t>Clap de cinéma</t>
+          <t>Spatule à la main</t>
         </is>
       </c>
       <c r="M191" s="5" t="inlineStr">
         <is>
-          <t>portraits/86-benoit-larouche-web.webp</t>
+          <t>portraits/186-stephane-bosse-web.webp</t>
         </is>
       </c>
       <c r="N191" s="5" t="inlineStr">
         <is>
-          <t>Larouche</t>
+          <t>Bossé</t>
         </is>
       </c>
       <c r="O191" s="5" t="n"/>
       <c r="P191" s="5" t="inlineStr">
         <is>
-          <t>Prof d’Antoine Lefèvre</t>
+          <t>Frère de Gaétan Bossé — conjoint de Marie-Ève Boucher</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Camille Lefèvre</t>
+          <t>Valentina Rojas</t>
         </is>
       </c>
       <c r="B192" s="2" t="n"/>
@@ -14289,138 +14297,142 @@
         </is>
       </c>
       <c r="D192" s="3" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>Étudiante en communications (UQAC)</t>
+          <t>Épicière — produits latino-américains</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>1127, Rue Saint-Dominique</t>
+          <t>318, Rue Bossé</t>
         </is>
       </c>
       <c r="H192" s="4" t="n">
-        <v>48.4214</v>
+        <v>48.4245</v>
       </c>
       <c r="I192" s="4" t="n">
-        <v>-71.24469999999999</v>
+        <v>-71.07585</v>
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>Carré brun, appareil photo</t>
+          <t>Longs cheveux noirs, anneaux dorés</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>Manteau friperie</t>
+          <t>Tablier vert sur chandail</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
-          <t>Pentax vintage</t>
+          <t>Caisse de plantains</t>
         </is>
       </c>
       <c r="M192" s="2" t="inlineStr">
         <is>
-          <t>portraits/65-camille-lefevre-web.webp</t>
+          <t>portraits/189-valentina-rojas-web.webp</t>
         </is>
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>Lefèvre</t>
+          <t>Rojas</t>
         </is>
       </c>
       <c r="O192" s="2" t="n"/>
       <c r="P192" s="2" t="inlineStr">
         <is>
-          <t>Sœur d’Antoine Lefèvre</t>
+          <t>Célibataire</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="5" t="inlineStr">
         <is>
-          <t>Dany Aubin</t>
-        </is>
-      </c>
-      <c r="B193" s="5" t="n"/>
+          <t>Vittorio Santini</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Don Vittorio</t>
+        </is>
+      </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D193" s="6" t="n">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="E193" s="5" t="inlineStr">
         <is>
-          <t>Soudeur</t>
+          <t>Homme d’affaires — restauration et bars</t>
         </is>
       </c>
       <c r="F193" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G193" s="5" t="inlineStr">
         <is>
-          <t>2147, Boulevard Harvey</t>
+          <t>200, Rue Racine Est</t>
         </is>
       </c>
       <c r="H193" s="7" t="n">
-        <v>48.41282</v>
+        <v>48.4281</v>
       </c>
       <c r="I193" s="7" t="n">
-        <v>-71.24145</v>
+        <v>-71.0545</v>
       </c>
       <c r="J193" s="5" t="inlineStr">
         <is>
-          <t>Brûlé de soudeur, casque relevé</t>
+          <t>Cheveux argentés gominés, chevalière</t>
         </is>
       </c>
       <c r="K193" s="5" t="inlineStr">
         <is>
-          <t>Manteau de soudeur</t>
+          <t>Manteau noir</t>
         </is>
       </c>
       <c r="L193" s="5" t="inlineStr">
         <is>
-          <t>Masque de soudure</t>
+          <t>Chevalière en or</t>
         </is>
       </c>
       <c r="M193" s="5" t="inlineStr">
         <is>
-          <t>portraits/66-dany-aubin-web.webp</t>
+          <t>portraits/151-vittorio-santini-web.webp</t>
         </is>
       </c>
       <c r="N193" s="5" t="inlineStr">
         <is>
-          <t>Aubin</t>
+          <t>Santini</t>
         </is>
       </c>
       <c r="O193" s="5" t="n"/>
       <c r="P193" s="5" t="inlineStr">
         <is>
-          <t>Frère de Sam Aubin</t>
+          <t>Époux de Maria — tient Dévon à distance</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Fernand Lavoie</t>
+          <t>William Lavoie</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Ti-Fer</t>
+          <t>Will</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
@@ -14429,47 +14441,47 @@
         </is>
       </c>
       <c r="D194" s="3" t="n">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>Retraité — ex-opérateur de cuves à l’aluminerie</t>
+          <t>Cuisinier — bistro du centre-ville</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>2131, Rue Davis</t>
+          <t>318, Rue Saint-Vallier</t>
         </is>
       </c>
       <c r="H194" s="4" t="n">
-        <v>48.4244</v>
+        <v>48.4263</v>
       </c>
       <c r="I194" s="4" t="n">
-        <v>-71.18225</v>
+        <v>-71.05034999999999</v>
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>Casquette plate, mains larges</t>
+          <t>Bandana, bras tatoué</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>Veste de laine à carreaux</t>
+          <t>Veste de cuisine ouverte</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>Pipe éteinte</t>
+          <t>Vapoteuse</t>
         </is>
       </c>
       <c r="M194" s="2" t="inlineStr">
         <is>
-          <t>portraits/190-fernand-lavoie-web.webp</t>
+          <t>portraits/206-william-lavoie-web.webp</t>
         </is>
       </c>
       <c r="N194" s="2" t="inlineStr">
@@ -14479,24 +14491,24 @@
       </c>
       <c r="O194" s="2" t="inlineStr">
         <is>
-          <t>Arvida</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>Père d’Audrey Lavoie — cousin éloigné de Mathieu Lavoie</t>
+          <t>Cousin de JP — colocataire d’Emma Boucher et Moussa Diallo</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="5" t="inlineStr">
         <is>
-          <t>Gérald Tremblay</t>
+          <t>Éric Simard</t>
         </is>
       </c>
       <c r="B195" s="5" t="inlineStr">
         <is>
-          <t>Le Syndic</t>
+          <t>Ti-Eric</t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
@@ -14505,83 +14517,83 @@
         </is>
       </c>
       <c r="D195" s="6" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="E195" s="5" t="inlineStr">
         <is>
-          <t>Délégué syndical — aluminerie</t>
+          <t>Étudiant — Cégep de Chicoutimi</t>
         </is>
       </c>
       <c r="F195" s="5" t="inlineStr">
         <is>
-          <t>Jonquière</t>
+          <t>Chicoutimi</t>
         </is>
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>3324, Rue Price</t>
+          <t>1184, Boulevard Talbot</t>
         </is>
       </c>
       <c r="H195" s="7" t="n">
-        <v>48.4258</v>
+        <v>48.3984</v>
       </c>
       <c r="I195" s="7" t="n">
-        <v>-71.24039999999999</v>
+        <v>-71.06740000000001</v>
       </c>
       <c r="J195" s="5" t="inlineStr">
         <is>
-          <t>Manteau de travail, épinglette</t>
+          <t>Casquette, jeans</t>
         </is>
       </c>
       <c r="K195" s="5" t="inlineStr">
         <is>
-          <t>Manteau d’usine</t>
+          <t>Hoodie cégep</t>
         </is>
       </c>
       <c r="L195" s="5" t="inlineStr">
         <is>
-          <t>Cartable de griefs</t>
+          <t>Skateboard</t>
         </is>
       </c>
       <c r="M195" s="5" t="inlineStr">
         <is>
-          <t>portraits/137-gerald-tremblay-web.webp</t>
+          <t>portraits/100-eric-simard-web.webp</t>
         </is>
       </c>
       <c r="N195" s="5" t="inlineStr">
         <is>
-          <t>Tremblay</t>
-        </is>
-      </c>
-      <c r="O195" s="5" t="inlineStr">
-        <is>
-          <t>syndicat</t>
-        </is>
-      </c>
+          <t>Chen</t>
+        </is>
+      </c>
+      <c r="O195" s="5" t="n"/>
       <c r="P195" s="5" t="inlineStr">
         <is>
-          <t>Collègue de Mathieu Lavoie</t>
+          <t>Colocataire de Justin Chen</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Jade Boivin</t>
-        </is>
-      </c>
-      <c r="B196" s="2" t="n"/>
+          <t>Anthony Simard</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Tony Steak</t>
+        </is>
+      </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D196" s="3" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>Élève du primaire — patineuse artistique</t>
+          <t>Apprenti boucher — boucherie familiale</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -14591,65 +14603,73 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>2350, Rue Sainte-Famille</t>
+          <t>2216, Rue Saint-Joseph</t>
         </is>
       </c>
       <c r="H196" s="4" t="n">
-        <v>48.4293</v>
+        <v>48.42405</v>
       </c>
       <c r="I196" s="4" t="n">
-        <v>-71.23480000000001</v>
+        <v>-71.2316</v>
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>Chignon serré, sourire édenté</t>
+          <t>Cheveux ras, pansement au doigt</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>Veston d’entraînement mauve</t>
+          <t>Sarrau blanc, tablier rayé</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
-          <t>Protège-lames</t>
+          <t>Couteau à désosser</t>
         </is>
       </c>
       <c r="M196" s="2" t="inlineStr">
         <is>
-          <t>portraits/183-jade-boivin-web.webp</t>
+          <t>portraits/212-anthony-simard-web.webp</t>
         </is>
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>Boivin</t>
-        </is>
-      </c>
-      <c r="O196" s="2" t="n"/>
+          <t>Simard</t>
+        </is>
+      </c>
+      <c r="O196" s="2" t="inlineStr">
+        <is>
+          <t>Kénogami</t>
+        </is>
+      </c>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>Nièce de France et Maxime Boivin</t>
+          <t>Fils de Karine Simard — frère de Léa — neveu de Nancy Simard</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="5" t="inlineStr">
         <is>
-          <t>Jean-Marc Fortin</t>
-        </is>
-      </c>
-      <c r="B197" s="5" t="n"/>
+          <t>Antoine Lefèvre</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Le Français</t>
+        </is>
+      </c>
       <c r="C197" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D197" s="6" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E197" s="5" t="inlineStr">
         <is>
-          <t>Directeur d’usine — Rio Tinto Arvida</t>
+          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
         </is>
       </c>
       <c r="F197" s="5" t="inlineStr">
@@ -14659,73 +14679,65 @@
       </c>
       <c r="G197" s="5" t="inlineStr">
         <is>
-          <t>1, Rue des Alumineries</t>
+          <t>1125, Rue Saint-Dominique</t>
         </is>
       </c>
       <c r="H197" s="7" t="n">
-        <v>48.4265</v>
+        <v>48.421279</v>
       </c>
       <c r="I197" s="7" t="n">
-        <v>-71.182</v>
+        <v>-71.244586</v>
       </c>
       <c r="J197" s="5" t="inlineStr">
         <is>
-          <t>Cheveux argentés, manteau</t>
+          <t>Barbe hipster</t>
         </is>
       </c>
       <c r="K197" s="5" t="inlineStr">
         <is>
-          <t>Manteau et casque blanc</t>
+          <t>Friperie, caméra Sony</t>
         </is>
       </c>
       <c r="L197" s="5" t="inlineStr">
         <is>
-          <t>Casque sous le bras</t>
+          <t>Veut docu raw</t>
         </is>
       </c>
       <c r="M197" s="5" t="inlineStr">
         <is>
-          <t>portraits/125-jean-marc-fortin-web.webp</t>
+          <t>portraits/20-antoine-lefevre-web.webp</t>
         </is>
       </c>
       <c r="N197" s="5" t="inlineStr">
         <is>
-          <t>Fortin</t>
-        </is>
-      </c>
-      <c r="O197" s="5" t="inlineStr">
-        <is>
-          <t>industrie</t>
-        </is>
-      </c>
+          <t>Lefèvre</t>
+        </is>
+      </c>
+      <c r="O197" s="5" t="n"/>
       <c r="P197" s="5" t="inlineStr">
         <is>
-          <t>Patron de Mathieu Lavoie et Nicolas Gagné</t>
+          <t>Frère de Camille</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Ludovic Larouche</t>
-        </is>
-      </c>
-      <c r="B198" s="2" t="inlineStr">
-        <is>
-          <t>Ludo</t>
-        </is>
-      </c>
+          <t>Audrey Lavoie</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="n"/>
       <c r="C198" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D198" s="3" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+          <t>Apprentie électricienne — aluminerie Rio Tinto Arvida</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
@@ -14735,69 +14747,69 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>2507, Rue Saint-Hubert</t>
+          <t>2135, Rue Davis</t>
         </is>
       </c>
       <c r="H198" s="4" t="n">
-        <v>48.41615</v>
+        <v>48.42455</v>
       </c>
       <c r="I198" s="4" t="n">
-        <v>-71.25285</v>
+        <v>-71.18219999999999</v>
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>Boucles, lunettes rondes</t>
+          <t>Tresse blonde, lunettes de sécurité</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
-          <t>Veste en velours côtelé</t>
+          <t>Manteau orange haute visibilité</t>
         </is>
       </c>
       <c r="L198" s="2" t="inlineStr">
         <is>
-          <t>Caméscope à l’épaule</t>
+          <t>Glacière à lunch</t>
         </is>
       </c>
       <c r="M198" s="2" t="inlineStr">
         <is>
-          <t>portraits/182-ludovic-larouche-web.webp</t>
+          <t>portraits/191-audrey-lavoie-web.webp</t>
         </is>
       </c>
       <c r="N198" s="2" t="inlineStr">
         <is>
-          <t>Larouche</t>
-        </is>
-      </c>
-      <c r="O198" s="2" t="n"/>
+          <t>Lavoie</t>
+        </is>
+      </c>
+      <c r="O198" s="2" t="inlineStr">
+        <is>
+          <t>Arvida</t>
+        </is>
+      </c>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>Fils de Benoit Larouche</t>
+          <t>Fille de Fernand Lavoie — collègue de Nicolas Gagné</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="5" t="inlineStr">
         <is>
-          <t>Marc Picard</t>
-        </is>
-      </c>
-      <c r="B199" s="5" t="inlineStr">
-        <is>
-          <t>L’Arpenteur</t>
-        </is>
-      </c>
+          <t>Benoit Larouche</t>
+        </is>
+      </c>
+      <c r="B199" s="5" t="n"/>
       <c r="C199" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D199" s="6" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E199" s="5" t="inlineStr">
         <is>
-          <t>Arpenteur-géomètre</t>
+          <t>Enseignant — Cégep de Jonquière (ATM)</t>
         </is>
       </c>
       <c r="F199" s="5" t="inlineStr">
@@ -14807,69 +14819,65 @@
       </c>
       <c r="G199" s="5" t="inlineStr">
         <is>
-          <t>1220, Rue du Vieux-Pont</t>
+          <t>2505, Rue Saint-Hubert</t>
         </is>
       </c>
       <c r="H199" s="7" t="n">
-        <v>48.4113</v>
+        <v>48.416</v>
       </c>
       <c r="I199" s="7" t="n">
-        <v>-71.2679</v>
+        <v>-71.253</v>
       </c>
       <c r="J199" s="5" t="inlineStr">
         <is>
-          <t>Innu de Mashteuiatsh, cheveux longs attachés</t>
+          <t>Lunettes, barbe grise</t>
         </is>
       </c>
       <c r="K199" s="5" t="inlineStr">
         <is>
-          <t>Dossard orange sur polar</t>
+          <t>Chemise et cardigan</t>
         </is>
       </c>
       <c r="L199" s="5" t="inlineStr">
         <is>
-          <t>Station totale sur trépied</t>
+          <t>Clap de cinéma</t>
         </is>
       </c>
       <c r="M199" s="5" t="inlineStr">
         <is>
-          <t>portraits/193-marc-picard-web.webp</t>
+          <t>portraits/86-benoit-larouche-web.webp</t>
         </is>
       </c>
       <c r="N199" s="5" t="inlineStr">
         <is>
-          <t>Picard</t>
+          <t>Larouche</t>
         </is>
       </c>
       <c r="O199" s="5" t="n"/>
       <c r="P199" s="5" t="inlineStr">
         <is>
-          <t>Célibataire — croise William McKenzie</t>
+          <t>Prof d’Antoine Lefèvre</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Mathieu Lavoie</t>
-        </is>
-      </c>
-      <c r="B200" s="2" t="inlineStr">
-        <is>
-          <t>Mat</t>
-        </is>
-      </c>
+          <t>Camille Lefèvre</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="n"/>
       <c r="C200" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D200" s="3" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>Technicien à l'aluminerie Rio Tinto — Arvida</t>
+          <t>Étudiante en communications (UQAC)</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
@@ -14879,55 +14887,51 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>3320, Rue Price</t>
+          <t>1127, Rue Saint-Dominique</t>
         </is>
       </c>
       <c r="H200" s="4" t="n">
-        <v>48.425907</v>
+        <v>48.4214</v>
       </c>
       <c r="I200" s="4" t="n">
-        <v>-71.240752</v>
+        <v>-71.24469999999999</v>
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>Propre, polo Rio Tinto</t>
+          <t>Carré brun, appareil photo</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
         <is>
-          <t>Polo Rio Tinto</t>
+          <t>Manteau friperie</t>
         </is>
       </c>
       <c r="L200" s="2" t="inlineStr">
         <is>
-          <t>Boîte à lunch</t>
+          <t>Pentax vintage</t>
         </is>
       </c>
       <c r="M200" s="2" t="inlineStr">
         <is>
-          <t>portraits/35-mathieu-lavoie-web.webp</t>
+          <t>portraits/65-camille-lefevre-web.webp</t>
         </is>
       </c>
       <c r="N200" s="2" t="inlineStr">
         <is>
-          <t>Lavoie</t>
-        </is>
-      </c>
-      <c r="O200" s="2" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
+          <t>Lefèvre</t>
+        </is>
+      </c>
+      <c r="O200" s="2" t="n"/>
       <c r="P200" s="2" t="inlineStr">
         <is>
-          <t>Frère aîné de JP</t>
+          <t>Sœur d’Antoine Lefèvre</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="5" t="inlineStr">
         <is>
-          <t>Mélissa Harvey</t>
+          <t>Dany Aubin</t>
         </is>
       </c>
       <c r="B201" s="5" t="n"/>
@@ -14937,11 +14941,11 @@
         </is>
       </c>
       <c r="D201" s="6" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E201" s="5" t="inlineStr">
         <is>
-          <t>Étudiante en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+          <t>Soudeur</t>
         </is>
       </c>
       <c r="F201" s="5" t="inlineStr">
@@ -14951,56 +14955,56 @@
       </c>
       <c r="G201" s="5" t="inlineStr">
         <is>
-          <t>1129, Rue Saint-Dominique</t>
+          <t>2147, Boulevard Harvey</t>
         </is>
       </c>
       <c r="H201" s="7" t="n">
-        <v>48.42135</v>
+        <v>48.41282</v>
       </c>
       <c r="I201" s="7" t="n">
-        <v>-71.24464999999999</v>
+        <v>-71.24145</v>
       </c>
       <c r="J201" s="5" t="inlineStr">
         <is>
-          <t>Chignon brouillon, manteau friperie</t>
+          <t>Brûlé de soudeur, casque relevé</t>
         </is>
       </c>
       <c r="K201" s="5" t="inlineStr">
         <is>
-          <t>Manteau friperie</t>
+          <t>Manteau de soudeur</t>
         </is>
       </c>
       <c r="L201" s="5" t="inlineStr">
         <is>
-          <t>Perche micro</t>
+          <t>Masque de soudure</t>
         </is>
       </c>
       <c r="M201" s="5" t="inlineStr">
         <is>
-          <t>portraits/110-melissa-harvey-web.webp</t>
+          <t>portraits/66-dany-aubin-web.webp</t>
         </is>
       </c>
       <c r="N201" s="5" t="inlineStr">
         <is>
-          <t>Harvey</t>
+          <t>Aubin</t>
         </is>
       </c>
       <c r="O201" s="5" t="n"/>
       <c r="P201" s="5" t="inlineStr">
         <is>
-          <t>Nièce de François Harvey</t>
+          <t>Frère de Sam Aubin</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Nancy Simard</t>
+          <t>Fernand Lavoie</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>Nancy Ciseaux</t>
+          <t>Ti-Fer</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
@@ -15009,11 +15013,11 @@
         </is>
       </c>
       <c r="D202" s="3" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Coiffeuse — propriétaire de salon</t>
+          <t>Retraité — ex-opérateur de cuves à l’aluminerie</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
@@ -15023,69 +15027,73 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>3812, Rue Saint-Hubert</t>
+          <t>2131, Rue Davis</t>
         </is>
       </c>
       <c r="H202" s="4" t="n">
-        <v>48.41605</v>
+        <v>48.4244</v>
       </c>
       <c r="I202" s="4" t="n">
-        <v>-71.2453</v>
+        <v>-71.18225</v>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Blond platine, grosses boucles d’oreilles</t>
+          <t>Casquette plate, mains larges</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Sarrau noir de coiffeuse</t>
+          <t>Veste de laine à carreaux</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
         <is>
-          <t>Ciseaux et peigne</t>
+          <t>Pipe éteinte</t>
         </is>
       </c>
       <c r="M202" s="2" t="inlineStr">
         <is>
-          <t>portraits/192-nancy-simard-web.webp</t>
+          <t>portraits/190-fernand-lavoie-web.webp</t>
         </is>
       </c>
       <c r="N202" s="2" t="inlineStr">
         <is>
-          <t>Simard</t>
+          <t>Lavoie</t>
         </is>
       </c>
       <c r="O202" s="2" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>Arvida</t>
         </is>
       </c>
       <c r="P202" s="2" t="inlineStr">
         <is>
-          <t>Célibataire — voisine de Benoit Larouche</t>
+          <t>Père d’Audrey Lavoie — cousin éloigné de Mathieu Lavoie</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="5" t="inlineStr">
         <is>
-          <t>Nicolas Gagné</t>
-        </is>
-      </c>
-      <c r="B203" s="5" t="n"/>
+          <t>Gérald Tremblay</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>Le Syndic</t>
+        </is>
+      </c>
       <c r="C203" s="6" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D203" s="6" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E203" s="5" t="inlineStr">
         <is>
-          <t>Technicien — aluminerie Rio Tinto Arvida</t>
+          <t>Délégué syndical — aluminerie</t>
         </is>
       </c>
       <c r="F203" s="5" t="inlineStr">
@@ -15095,43 +15103,43 @@
       </c>
       <c r="G203" s="5" t="inlineStr">
         <is>
-          <t>3322, Rue Price</t>
+          <t>3324, Rue Price</t>
         </is>
       </c>
       <c r="H203" s="7" t="n">
-        <v>48.426</v>
+        <v>48.4258</v>
       </c>
       <c r="I203" s="7" t="n">
-        <v>-71.2405</v>
+        <v>-71.24039999999999</v>
       </c>
       <c r="J203" s="5" t="inlineStr">
         <is>
-          <t>Propre, lunettes de sécurité</t>
+          <t>Manteau de travail, épinglette</t>
         </is>
       </c>
       <c r="K203" s="5" t="inlineStr">
         <is>
-          <t>Polo Rio Tinto</t>
+          <t>Manteau d’usine</t>
         </is>
       </c>
       <c r="L203" s="5" t="inlineStr">
         <is>
-          <t>Casque blanc</t>
+          <t>Cartable de griefs</t>
         </is>
       </c>
       <c r="M203" s="5" t="inlineStr">
         <is>
-          <t>portraits/94-nicolas-gagne-web.webp</t>
+          <t>portraits/137-gerald-tremblay-web.webp</t>
         </is>
       </c>
       <c r="N203" s="5" t="inlineStr">
         <is>
-          <t>Gagné</t>
+          <t>Tremblay</t>
         </is>
       </c>
       <c r="O203" s="5" t="inlineStr">
         <is>
-          <t>Arvida</t>
+          <t>syndicat</t>
         </is>
       </c>
       <c r="P203" s="5" t="inlineStr">
@@ -15143,25 +15151,21 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Sam Aubin</t>
-        </is>
-      </c>
-      <c r="B204" s="2" t="inlineStr">
-        <is>
-          <t>Ink</t>
-        </is>
-      </c>
+          <t>Jade Boivin</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="n"/>
       <c r="C204" s="3" t="inlineStr">
         <is>
           <t>Humain</t>
         </is>
       </c>
       <c r="D204" s="3" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>Tatoueur</t>
+          <t>Élève du primaire — patineuse artistique</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
@@ -15171,49 +15175,777 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>2145, Boulevard Harvey</t>
+          <t>2350, Rue Sainte-Famille</t>
         </is>
       </c>
       <c r="H204" s="4" t="n">
-        <v>48.412694</v>
+        <v>48.4293</v>
       </c>
       <c r="I204" s="4" t="n">
-        <v>-71.241325</v>
+        <v>-71.23480000000001</v>
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>Cheveux bleus, full tattoos</t>
+          <t>Chignon serré, sourire édenté</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>Tablier noir</t>
+          <t>Veston d’entraînement mauve</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
         <is>
-          <t>Efface tattoos gang</t>
+          <t>Protège-lames</t>
         </is>
       </c>
       <c r="M204" s="2" t="inlineStr">
         <is>
-          <t>portraits/24-sam-aubin-web.webp</t>
+          <t>portraits/183-jade-boivin-web.webp</t>
         </is>
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>Aubin</t>
+          <t>Boivin</t>
         </is>
       </c>
       <c r="O204" s="2" t="n"/>
       <c r="P204" s="2" t="inlineStr">
         <is>
+          <t>Nièce de France et Maxime Boivin</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="inlineStr">
+        <is>
+          <t>Jean-Marc Fortin</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="n"/>
+      <c r="C205" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D205" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>Directeur d’usine — Rio Tinto Arvida</t>
+        </is>
+      </c>
+      <c r="F205" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G205" s="5" t="inlineStr">
+        <is>
+          <t>1, Rue des Alumineries</t>
+        </is>
+      </c>
+      <c r="H205" s="7" t="n">
+        <v>48.4265</v>
+      </c>
+      <c r="I205" s="7" t="n">
+        <v>-71.182</v>
+      </c>
+      <c r="J205" s="5" t="inlineStr">
+        <is>
+          <t>Cheveux argentés, manteau</t>
+        </is>
+      </c>
+      <c r="K205" s="5" t="inlineStr">
+        <is>
+          <t>Manteau et casque blanc</t>
+        </is>
+      </c>
+      <c r="L205" s="5" t="inlineStr">
+        <is>
+          <t>Casque sous le bras</t>
+        </is>
+      </c>
+      <c r="M205" s="5" t="inlineStr">
+        <is>
+          <t>portraits/125-jean-marc-fortin-web.webp</t>
+        </is>
+      </c>
+      <c r="N205" s="5" t="inlineStr">
+        <is>
+          <t>Fortin</t>
+        </is>
+      </c>
+      <c r="O205" s="5" t="inlineStr">
+        <is>
+          <t>industrie</t>
+        </is>
+      </c>
+      <c r="P205" s="5" t="inlineStr">
+        <is>
+          <t>Patron de Mathieu Lavoie et Nicolas Gagné</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Karine Simard</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Coach K</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>Enseignante d’éducation physique — entraîneuse de natation</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>2216, Rue Saint-Joseph</t>
+        </is>
+      </c>
+      <c r="H206" s="4" t="n">
+        <v>48.42395</v>
+      </c>
+      <c r="I206" s="4" t="n">
+        <v>-71.23180000000001</v>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>Athlétique, queue de cheval blonde</t>
+        </is>
+      </c>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>Veste de survêtement marine</t>
+        </is>
+      </c>
+      <c r="L206" s="2" t="inlineStr">
+        <is>
+          <t>Chronomètre</t>
+        </is>
+      </c>
+      <c r="M206" s="2" t="inlineStr">
+        <is>
+          <t>portraits/213-karine-simard-web.webp</t>
+        </is>
+      </c>
+      <c r="N206" s="2" t="inlineStr">
+        <is>
+          <t>Simard</t>
+        </is>
+      </c>
+      <c r="O206" s="2" t="inlineStr">
+        <is>
+          <t>Kénogami</t>
+        </is>
+      </c>
+      <c r="P206" s="2" t="inlineStr">
+        <is>
+          <t>Mère de Léa et Anthony — sœur de Nancy Simard</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>Ludovic Larouche</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>Ludo</t>
+        </is>
+      </c>
+      <c r="C207" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D207" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>Étudiant en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+        </is>
+      </c>
+      <c r="F207" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G207" s="5" t="inlineStr">
+        <is>
+          <t>2507, Rue Saint-Hubert</t>
+        </is>
+      </c>
+      <c r="H207" s="7" t="n">
+        <v>48.41615</v>
+      </c>
+      <c r="I207" s="7" t="n">
+        <v>-71.25285</v>
+      </c>
+      <c r="J207" s="5" t="inlineStr">
+        <is>
+          <t>Boucles, lunettes rondes</t>
+        </is>
+      </c>
+      <c r="K207" s="5" t="inlineStr">
+        <is>
+          <t>Veste en velours côtelé</t>
+        </is>
+      </c>
+      <c r="L207" s="5" t="inlineStr">
+        <is>
+          <t>Caméscope à l’épaule</t>
+        </is>
+      </c>
+      <c r="M207" s="5" t="inlineStr">
+        <is>
+          <t>portraits/182-ludovic-larouche-web.webp</t>
+        </is>
+      </c>
+      <c r="N207" s="5" t="inlineStr">
+        <is>
+          <t>Larouche</t>
+        </is>
+      </c>
+      <c r="O207" s="5" t="n"/>
+      <c r="P207" s="5" t="inlineStr">
+        <is>
+          <t>Fils de Benoit Larouche</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Léa Simard</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="n"/>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>Élève du secondaire — nageuse de compétition</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>2216, Rue Saint-Joseph</t>
+        </is>
+      </c>
+      <c r="H208" s="4" t="n">
+        <v>48.424</v>
+      </c>
+      <c r="I208" s="4" t="n">
+        <v>-71.2317</v>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>Cheveux mouillés, l’air déterminé</t>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>Serviette sur les épaules</t>
+        </is>
+      </c>
+      <c r="L208" s="2" t="inlineStr">
+        <is>
+          <t>Lunettes de piscine sur le front</t>
+        </is>
+      </c>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t>portraits/211-lea-simard-web.webp</t>
+        </is>
+      </c>
+      <c r="N208" s="2" t="inlineStr">
+        <is>
+          <t>Simard</t>
+        </is>
+      </c>
+      <c r="O208" s="2" t="inlineStr">
+        <is>
+          <t>Kénogami</t>
+        </is>
+      </c>
+      <c r="P208" s="2" t="inlineStr">
+        <is>
+          <t>Fille de Karine Simard — sœur d’Anthony</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="inlineStr">
+        <is>
+          <t>Marc Picard</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>L’Arpenteur</t>
+        </is>
+      </c>
+      <c r="C209" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D209" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>Arpenteur-géomètre</t>
+        </is>
+      </c>
+      <c r="F209" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G209" s="5" t="inlineStr">
+        <is>
+          <t>1220, Rue du Vieux-Pont</t>
+        </is>
+      </c>
+      <c r="H209" s="7" t="n">
+        <v>48.4113</v>
+      </c>
+      <c r="I209" s="7" t="n">
+        <v>-71.2679</v>
+      </c>
+      <c r="J209" s="5" t="inlineStr">
+        <is>
+          <t>Innu de Mashteuiatsh, cheveux longs attachés</t>
+        </is>
+      </c>
+      <c r="K209" s="5" t="inlineStr">
+        <is>
+          <t>Dossard orange sur polar</t>
+        </is>
+      </c>
+      <c r="L209" s="5" t="inlineStr">
+        <is>
+          <t>Station totale sur trépied</t>
+        </is>
+      </c>
+      <c r="M209" s="5" t="inlineStr">
+        <is>
+          <t>portraits/193-marc-picard-web.webp</t>
+        </is>
+      </c>
+      <c r="N209" s="5" t="inlineStr">
+        <is>
+          <t>Picard</t>
+        </is>
+      </c>
+      <c r="O209" s="5" t="n"/>
+      <c r="P209" s="5" t="inlineStr">
+        <is>
+          <t>Célibataire — croise William McKenzie</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>Mathieu Lavoie</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>Technicien à l'aluminerie Rio Tinto — Arvida</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>3320, Rue Price</t>
+        </is>
+      </c>
+      <c r="H210" s="4" t="n">
+        <v>48.425907</v>
+      </c>
+      <c r="I210" s="4" t="n">
+        <v>-71.240752</v>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>Propre, polo Rio Tinto</t>
+        </is>
+      </c>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>Polo Rio Tinto</t>
+        </is>
+      </c>
+      <c r="L210" s="2" t="inlineStr">
+        <is>
+          <t>Boîte à lunch</t>
+        </is>
+      </c>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t>portraits/35-mathieu-lavoie-web.webp</t>
+        </is>
+      </c>
+      <c r="N210" s="2" t="inlineStr">
+        <is>
+          <t>Lavoie</t>
+        </is>
+      </c>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="P210" s="2" t="inlineStr">
+        <is>
+          <t>Frère aîné de JP</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="inlineStr">
+        <is>
+          <t>Mélissa Harvey</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="n"/>
+      <c r="C211" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D211" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>Étudiante en cinéma et télévision (Cégep de Jonquière — ATM)</t>
+        </is>
+      </c>
+      <c r="F211" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>1129, Rue Saint-Dominique</t>
+        </is>
+      </c>
+      <c r="H211" s="7" t="n">
+        <v>48.42135</v>
+      </c>
+      <c r="I211" s="7" t="n">
+        <v>-71.24464999999999</v>
+      </c>
+      <c r="J211" s="5" t="inlineStr">
+        <is>
+          <t>Chignon brouillon, manteau friperie</t>
+        </is>
+      </c>
+      <c r="K211" s="5" t="inlineStr">
+        <is>
+          <t>Manteau friperie</t>
+        </is>
+      </c>
+      <c r="L211" s="5" t="inlineStr">
+        <is>
+          <t>Perche micro</t>
+        </is>
+      </c>
+      <c r="M211" s="5" t="inlineStr">
+        <is>
+          <t>portraits/110-melissa-harvey-web.webp</t>
+        </is>
+      </c>
+      <c r="N211" s="5" t="inlineStr">
+        <is>
+          <t>Harvey</t>
+        </is>
+      </c>
+      <c r="O211" s="5" t="n"/>
+      <c r="P211" s="5" t="inlineStr">
+        <is>
+          <t>Nièce de François Harvey</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>Nancy Simard</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Nancy Ciseaux</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>Coiffeuse — propriétaire de salon</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>3812, Rue Saint-Hubert</t>
+        </is>
+      </c>
+      <c r="H212" s="4" t="n">
+        <v>48.41605</v>
+      </c>
+      <c r="I212" s="4" t="n">
+        <v>-71.2453</v>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>Blond platine, grosses boucles d’oreilles</t>
+        </is>
+      </c>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
+          <t>Sarrau noir de coiffeuse</t>
+        </is>
+      </c>
+      <c r="L212" s="2" t="inlineStr">
+        <is>
+          <t>Ciseaux et peigne</t>
+        </is>
+      </c>
+      <c r="M212" s="2" t="inlineStr">
+        <is>
+          <t>portraits/192-nancy-simard-web.webp</t>
+        </is>
+      </c>
+      <c r="N212" s="2" t="inlineStr">
+        <is>
+          <t>Simard</t>
+        </is>
+      </c>
+      <c r="O212" s="2" t="inlineStr">
+        <is>
+          <t>salon</t>
+        </is>
+      </c>
+      <c r="P212" s="2" t="inlineStr">
+        <is>
+          <t>Célibataire — voisine de Benoit Larouche</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="5" t="inlineStr">
+        <is>
+          <t>Nicolas Gagné</t>
+        </is>
+      </c>
+      <c r="B213" s="5" t="n"/>
+      <c r="C213" s="6" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D213" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>Technicien — aluminerie Rio Tinto Arvida</t>
+        </is>
+      </c>
+      <c r="F213" s="5" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G213" s="5" t="inlineStr">
+        <is>
+          <t>3322, Rue Price</t>
+        </is>
+      </c>
+      <c r="H213" s="7" t="n">
+        <v>48.426</v>
+      </c>
+      <c r="I213" s="7" t="n">
+        <v>-71.2405</v>
+      </c>
+      <c r="J213" s="5" t="inlineStr">
+        <is>
+          <t>Propre, lunettes de sécurité</t>
+        </is>
+      </c>
+      <c r="K213" s="5" t="inlineStr">
+        <is>
+          <t>Polo Rio Tinto</t>
+        </is>
+      </c>
+      <c r="L213" s="5" t="inlineStr">
+        <is>
+          <t>Casque blanc</t>
+        </is>
+      </c>
+      <c r="M213" s="5" t="inlineStr">
+        <is>
+          <t>portraits/94-nicolas-gagne-web.webp</t>
+        </is>
+      </c>
+      <c r="N213" s="5" t="inlineStr">
+        <is>
+          <t>Gagné</t>
+        </is>
+      </c>
+      <c r="O213" s="5" t="inlineStr">
+        <is>
+          <t>Arvida</t>
+        </is>
+      </c>
+      <c r="P213" s="5" t="inlineStr">
+        <is>
+          <t>Collègue de Mathieu Lavoie</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>Sam Aubin</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Ink</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>Humain</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>Tatoueur</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>Jonquière</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>2145, Boulevard Harvey</t>
+        </is>
+      </c>
+      <c r="H214" s="4" t="n">
+        <v>48.412694</v>
+      </c>
+      <c r="I214" s="4" t="n">
+        <v>-71.241325</v>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>Cheveux bleus, full tattoos</t>
+        </is>
+      </c>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>Tablier noir</t>
+        </is>
+      </c>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t>Efface tattoos gang</t>
+        </is>
+      </c>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t>portraits/24-sam-aubin-web.webp</t>
+        </is>
+      </c>
+      <c r="N214" s="2" t="inlineStr">
+        <is>
+          <t>Aubin</t>
+        </is>
+      </c>
+      <c r="O214" s="2" t="n"/>
+      <c r="P214" s="2" t="inlineStr">
+        <is>
           <t>Frère de Dany</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P204"/>
+  <autoFilter ref="A1:P214"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15249,7 +15981,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>203 entrées · 16 colonnes · région du Saguenay (Québec)</t>
+          <t>213 entrées · 16 colonnes · région du Saguenay (Québec)</t>
         </is>
       </c>
     </row>

</xml_diff>